<commit_message>
chore: back up full workspace 2026-09-24
</commit_message>
<xml_diff>
--- a/watchlists/AI产业链.xlsx
+++ b/watchlists/AI产业链.xlsx
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E396"/>
+  <dimension ref="A1:E397"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6647,27 +6647,27 @@
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>半导体光掩膜版</t>
+          <t>晶圆硅片</t>
         </is>
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>688401</t>
+          <t>688432</t>
         </is>
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>路维光电</t>
+          <t>有研硅</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司平板显示与半导体掩膜版增长，G11、HTM、PSM等高端产品推进，AI算力、先进封装、AMOLED、Micro-LED等新兴领域带动高精度掩膜版需求；半导体占比仍需跟踪，主板块由泛光掩膜版收敛为高端掩膜版。</t>
+          <t>官方事实：主营半导体硅材料，产品含半导体硅抛光片、刻蚀设备用硅材料/零部件、区熔硅单晶及硅片，主要用于集成电路、分立/功率器件、传感器、光学器件及刻蚀设备；2026年7月并表安徽晶隆，增加8英寸硅外延片布局。AI关联为半导体需求的上游间接传导：2026年半年度报告提及AI驱动先进计算需求，但未披露具名AI客户、AI专项订单或可单独识别的AI收入。证据A：2026-08-14半年度报告第9、10、126页；2026-06-10、2026-07-07晶隆收购公告。</t>
         </is>
       </c>
       <c r="E213" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已复核；2026H1官方披露；AI客户/订单/独立收入=evidence_absent</t>
         </is>
       </c>
     </row>
@@ -6679,17 +6679,17 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>688138</t>
+          <t>688401</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>清溢光电</t>
+          <t>路维光电</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报显示公司主要从事掩膜版研发、设计、生产和销售，产品用于平板显示、半导体芯片、触控和电路板等；半导体国产替代和AI带动晶圆产能扩张构成间接受益，收入仍较依赖显示与综合掩膜版需求。</t>
+          <t>证据中强：2025年报披露公司平板显示与半导体掩膜版增长，G11、HTM、PSM等高端产品推进，AI算力、先进封装、AMOLED、Micro-LED等新兴领域带动高精度掩膜版需求；半导体占比仍需跟踪，主板块由泛光掩膜版收敛为高端掩膜版。</t>
         </is>
       </c>
       <c r="E214" s="6" t="inlineStr">
@@ -6706,17 +6706,17 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>688721</t>
+          <t>688138</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>龙图光罩</t>
+          <t>清溢光电</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司聚焦半导体掩模版，高端制程及关键客户开发持续推进、珠海工厂投产爬坡；但2025年净利润明显下滑，竞争、折旧和研发费用压制弹性，主板块保留半导体光掩膜版。</t>
+          <t>证据中：2025年报显示公司主要从事掩膜版研发、设计、生产和销售，产品用于平板显示、半导体芯片、触控和电路板等；半导体国产替代和AI带动晶圆产能扩张构成间接受益，收入仍较依赖显示与综合掩膜版需求。</t>
         </is>
       </c>
       <c r="E215" s="6" t="inlineStr">
@@ -6728,22 +6728,22 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>半导体前道设备</t>
+          <t>半导体光掩膜版</t>
         </is>
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>002371</t>
+          <t>688721</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>北方华创</t>
+          <t>龙图光罩</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露电子工艺装备收入高增，刻蚀、薄膜沉积、热处理、湿法清洗等主力设备放量，离子注入、电镀、混合键合等新品推进；MFC和清洗设备只是平台产品/子环节，合并删减重复行。</t>
+          <t>证据中强：2025年报披露公司聚焦半导体掩模版，高端制程及关键客户开发持续推进、珠海工厂投产爬坡；但2025年净利润明显下滑，竞争、折旧和研发费用压制弹性，主板块保留半导体光掩膜版。</t>
         </is>
       </c>
       <c r="E216" s="6" t="inlineStr">
@@ -6755,22 +6755,22 @@
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>离子注入设备/电子材料</t>
+          <t>半导体前道设备</t>
         </is>
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>600641</t>
+          <t>002371</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>先导基电</t>
+          <t>北方华创</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>证据A：原万业企业的主线为凯世通半导体离子注入设备；2026年7月以增资方式投资控股广东先导微电子，后续纳入合并范围，新增GaAs/Ge衬底、高纯金属、前驱体和电子特气等电子材料布局。其配套模拟审计报告假设先导微电子将InP业务相关资产、负债转至广东先锐，并自先导微电子模拟口径剔除相关资产、负债、收入、费用；因此不再按InP衬底资产或业绩处理。核心映射是晶圆厂半导体资本开支的间接受益，不属于800G/1.6T光互连的直接InP标的；风险是整合、融资及InP剥离交割边界。</t>
+          <t>证据强：2025年报披露电子工艺装备收入高增，刻蚀、薄膜沉积、热处理、湿法清洗等主力设备放量，离子注入、电镀、混合键合等新品推进；MFC和清洗设备只是平台产品/子环节，合并删减重复行。</t>
         </is>
       </c>
       <c r="E217" s="6" t="inlineStr">
@@ -6782,22 +6782,22 @@
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>刻蚀设备</t>
+          <t>离子注入设备/电子材料</t>
         </is>
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>688012</t>
+          <t>600641</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>中微公司</t>
+          <t>先导基电</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报/公开资料显示公司营收创新高，刻蚀设备为最大收入来源，LPCVD/ALD、MOCVD等新产品加速放量；先进封装TSV刻蚀等提供AI先进封装延伸，但主业和业绩弹性仍以刻蚀设备为核心。</t>
+          <t>证据A：原万业企业的主线为凯世通半导体离子注入设备；2026年7月以增资方式投资控股广东先导微电子，后续纳入合并范围，新增GaAs/Ge衬底、高纯金属、前驱体和电子特气等电子材料布局。其配套模拟审计报告假设先导微电子将InP业务相关资产、负债转至广东先锐，并自先导微电子模拟口径剔除相关资产、负债、收入、费用；因此不再按InP衬底资产或业绩处理。核心映射是晶圆厂半导体资本开支的间接受益，不属于800G/1.6T光互连的直接InP标的；风险是整合、融资及InP剥离交割边界。</t>
         </is>
       </c>
       <c r="E218" s="6" t="inlineStr">
@@ -6809,22 +6809,22 @@
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>薄膜沉积设备</t>
+          <t>刻蚀设备</t>
         </is>
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>688072</t>
+          <t>688012</t>
         </is>
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>拓荆科技</t>
+          <t>中微公司</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报显示PECVD、ALD、SACVD、HDPCVD等先进工艺设备在先进存储、先进逻辑规模化量产，在手订单较高；先进键合/三维集成设备已有突破但仍属扩展线，合并删减“先进封装设备”重复行。</t>
+          <t>证据强：2025年报/公开资料显示公司营收创新高，刻蚀设备为最大收入来源，LPCVD/ALD、MOCVD等新产品加速放量；先进封装TSV刻蚀等提供AI先进封装延伸，但主业和业绩弹性仍以刻蚀设备为核心。</t>
         </is>
       </c>
       <c r="E219" s="6" t="inlineStr">
@@ -6836,22 +6836,22 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>半导体清洗设备</t>
+          <t>薄膜沉积设备</t>
         </is>
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>688082</t>
+          <t>688072</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>盛美上海</t>
+          <t>拓荆科技</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露半导体清洗设备收入占比最高，清洗、电镀、立式炉管、先进封装湿法设备等多产品增长；先进封装湿法设备适配2.5D/3D封装和Chiplet但收入占比较小，合并删减“先进封装设备”重复行。</t>
+          <t>证据强：2025年报显示PECVD、ALD、SACVD、HDPCVD等先进工艺设备在先进存储、先进逻辑规模化量产，在手订单较高；先进键合/三维集成设备已有突破但仍属扩展线，合并删减“先进封装设备”重复行。</t>
         </is>
       </c>
       <c r="E220" s="6" t="inlineStr">
@@ -6863,22 +6863,22 @@
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>涂胶显影清洗设备</t>
+          <t>半导体清洗设备</t>
         </is>
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>688037</t>
+          <t>688082</t>
         </is>
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>芯源微</t>
+          <t>盛美上海</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报显示公司以光刻工序涂胶显影、单片式湿法清洗及先进封装湿法设备为主，前道晶圆加工与后道先进封装设备收入均增长；先进封装设备是AI/HBM链条延伸，主业弹性仍来自涂胶显影清洗平台，合并删减“先进封装设备”重复行。</t>
+          <t>证据强：2025年报披露半导体清洗设备收入占比最高，清洗、电镀、立式炉管、先进封装湿法设备等多产品增长；先进封装湿法设备适配2.5D/3D封装和Chiplet但收入占比较小，合并删减“先进封装设备”重复行。</t>
         </is>
       </c>
       <c r="E221" s="6" t="inlineStr">
@@ -6890,22 +6890,22 @@
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>CMP与减薄设备</t>
+          <t>涂胶显影清洗设备</t>
         </is>
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>688120</t>
+          <t>688037</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>华海清科</t>
+          <t>芯源微</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司CMP装备市场地位稳固，并突破先进封装减薄抛光设备、离子注入等新产品，CMP、减薄、划切、边抛等覆盖先进制程/先进封装/HBM需求；合并删减“晶圆减薄”重复行。</t>
+          <t>证据强：2025年报显示公司以光刻工序涂胶显影、单片式湿法清洗及先进封装湿法设备为主，前道晶圆加工与后道先进封装设备收入均增长；先进封装设备是AI/HBM链条延伸，主业弹性仍来自涂胶显影清洗平台，合并删减“先进封装设备”重复行。</t>
         </is>
       </c>
       <c r="E222" s="6" t="inlineStr">
@@ -6917,22 +6917,22 @@
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>封测切割减薄设备</t>
+          <t>CMP与减薄设备</t>
         </is>
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>300480</t>
+          <t>688120</t>
         </is>
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>光力科技</t>
+          <t>华海清科</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司半导体封测装备覆盖晶圆切割、封装体切割、晶圆减薄等环节，部分划切设备已在先进封装中批量应用；晶圆减薄和先进封装切割属于同一封测装备链，合并删减重复行。</t>
+          <t>证据强：2025年报披露公司CMP装备市场地位稳固，并突破先进封装减薄抛光设备、离子注入等新产品，CMP、减薄、划切、边抛等覆盖先进制程/先进封装/HBM需求；合并删减“晶圆减薄”重复行。</t>
         </is>
       </c>
       <c r="E223" s="6" t="inlineStr">
@@ -6944,22 +6944,22 @@
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>精密磨削设备</t>
+          <t>封测切割减薄设备</t>
         </is>
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>002903</t>
+          <t>300480</t>
         </is>
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>宇环数控</t>
+          <t>光力科技</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>证据弱中：2025年报显示公司主业仍为数控磨削抛光设备，全年亏损；晶圆减薄属于潜在高精密磨削应用，但半导体客户、订单和收入证据不足，原晶圆减薄降级为精密磨削设备并保留观察。</t>
+          <t>证据中强：2025年报披露公司半导体封测装备覆盖晶圆切割、封装体切割、晶圆减薄等环节，部分划切设备已在先进封装中批量应用；晶圆减薄和先进封装切割属于同一封测装备链，合并删减重复行。</t>
         </is>
       </c>
       <c r="E224" s="6" t="inlineStr">
@@ -6971,22 +6971,22 @@
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>半导体工艺温控</t>
+          <t>精密磨削设备</t>
         </is>
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>688652</t>
+          <t>002903</t>
         </is>
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>京仪装备</t>
+          <t>宇环数控</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司主营半导体专用温控设备，产品覆盖刻蚀、薄膜沉积、离子注入、清洗等核心制程，主要客户为国内头部晶圆厂和设备厂；工艺废气处理和AMHS为业务外延，合并进备注并删除重复行。</t>
+          <t>证据弱中：2025年报显示公司主业仍为数控磨削抛光设备，全年亏损；晶圆减薄属于潜在高精密磨削应用，但半导体客户、订单和收入证据不足，原晶圆减薄降级为精密磨削设备并保留观察。</t>
         </is>
       </c>
       <c r="E225" s="6" t="inlineStr">
@@ -6998,22 +6998,22 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>半导体真空泵</t>
+          <t>半导体工艺温控</t>
         </is>
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>002158</t>
+          <t>688652</t>
         </is>
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>汉钟精机</t>
+          <t>京仪装备</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报显示公司真空产品已应用于半导体、太阳能、锂电等领域，半导体真空泵是真实AI链条节点；工艺温控并非公司半导体主线，合并删减“半导体工艺温控”重复行。短期需跟踪半导体客户认证和收入占比。</t>
+          <t>证据强：2025年报披露公司主营半导体专用温控设备，产品覆盖刻蚀、薄膜沉积、离子注入、清洗等核心制程，主要客户为国内头部晶圆厂和设备厂；工艺废气处理和AMHS为业务外延，合并进备注并删除重复行。</t>
         </is>
       </c>
       <c r="E226" s="6" t="inlineStr">
@@ -7030,67 +7030,67 @@
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>暂无成熟A股纯标的</t>
+          <t>002158</t>
         </is>
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>高端干泵/涡轮分子泵纯标的不足</t>
+          <t>汉钟精机</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>高端半导体干泵和涡轮分子泵仍由Edwards、Pfeiffer、Ebara等海外厂商主导，A股除汉钟等配套外缺成熟纯标的。</t>
-        </is>
-      </c>
-      <c r="E227" s="6" t="n"/>
+          <t>证据中强：2025年报显示公司真空产品已应用于半导体、太阳能、锂电等领域，半导体真空泵是真实AI链条节点；工艺温控并非公司半导体主线，合并删减“半导体工艺温控”重复行。短期需跟踪半导体客户认证和收入占比。</t>
+        </is>
+      </c>
+      <c r="E227" s="6" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>半导体射频电源</t>
+          <t>半导体真空泵</t>
         </is>
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>300820</t>
+          <t>暂无成熟A股纯标的</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>英杰电气</t>
+          <t>高端干泵/涡轮分子泵纯标的不足</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报显示公司半导体等电子材料设备电源收入增长，射频电源、RPS远程等离子源等产品用于刻蚀/沉积/清洗等前道设备；公司不是离子注入设备商，合并删减“离子注入、RPS远程等离子源”重复行，主线收敛为半导体射频电源。</t>
-        </is>
-      </c>
-      <c r="E228" s="6" t="inlineStr">
-        <is>
-          <t>已处理</t>
-        </is>
-      </c>
+          <t>高端半导体干泵和涡轮分子泵仍由Edwards、Pfeiffer、Ebara等海外厂商主导，A股除汉钟等配套外缺成熟纯标的。</t>
+        </is>
+      </c>
+      <c r="E228" s="6" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>晶圆传输设备</t>
+          <t>半导体射频电源</t>
         </is>
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>300024</t>
+          <t>300820</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>机器人</t>
+          <t>英杰电气</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报显示公司半导体装备业务围绕晶圆搬运、真空机器人、EFEM、Load Port等产品，服务前道和后道设备厂商；原“半导体AMHS”过宽，主板块收敛为晶圆传输设备，AI受益来自国产半导体设备配套。</t>
+          <t>证据中强：2025年报显示公司半导体等电子材料设备电源收入增长，射频电源、RPS远程等离子源等产品用于刻蚀/沉积/清洗等前道设备；公司不是离子注入设备商，合并删减“离子注入、RPS远程等离子源”重复行，主线收敛为半导体射频电源。</t>
         </is>
       </c>
       <c r="E229" s="6" t="inlineStr">
@@ -7102,22 +7102,22 @@
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>半导体设备零部件</t>
+          <t>晶圆传输设备</t>
         </is>
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>688409</t>
+          <t>300024</t>
         </is>
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>富创精密</t>
+          <t>机器人</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司为半导体设备精密零部件平台，覆盖金属结构件、腔体、管路、模组等，并推进静电卡盘等高价值产品；静电卡盘是重要升级方向但不是唯一主线，合并删减“静电卡盘”重复行。</t>
+          <t>证据中强：2025年报显示公司半导体装备业务围绕晶圆搬运、真空机器人、EFEM、Load Port等产品，服务前道和后道设备厂商；原“半导体AMHS”过宽，主板块收敛为晶圆传输设备，AI受益来自国产半导体设备配套。</t>
         </is>
       </c>
       <c r="E230" s="6" t="inlineStr">
@@ -7129,27 +7129,27 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>半导体测试设备</t>
+          <t>半导体设备零部件</t>
         </is>
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>300604</t>
+          <t>688409</t>
         </is>
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>长川科技</t>
+          <t>富创精密</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报/公开资料显示公司已形成测试机、分选机、探针台、AOI等平台型产品矩阵，测试机成为核心收入来源，AI芯片复杂度提升、存储扩产和国产替代共同拉动高端测试设备需求；合并并删减“半导体测试分选机”重复行。2026-06-16 JPM补充：报告把GPU FT/SLT测试时间延长、TDP提升列为测试设备需求驱动，海外锚为Chroma；长川受益需验证高端SoC/SLT平台订单和AI客户收入，不泛化为所有测试机。</t>
+          <t>证据强：2025年报披露公司为半导体设备精密零部件平台，覆盖金属结构件、腔体、管路、模组等，并推进静电卡盘等高价值产品；静电卡盘是重要升级方向但不是唯一主线，合并删减“静电卡盘”重复行。</t>
         </is>
       </c>
       <c r="E231" s="6" t="inlineStr">
         <is>
-          <t>已处理；2026-06-16 JPM补充</t>
+          <t>已处理</t>
         </is>
       </c>
     </row>
@@ -7161,22 +7161,22 @@
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>688200</t>
+          <t>300604</t>
         </is>
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>华峰测控</t>
+          <t>长川科技</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司主营半导体自动化测试系统，收入和利润高增；AI相关弹性主要来自SoC/混合信号等高端测试平台放量与国产替代，现阶段仍以测试设备主业为核心，不单列为AI专用设备。</t>
+          <t>证据强：2025年报/公开资料显示公司已形成测试机、分选机、探针台、AOI等平台型产品矩阵，测试机成为核心收入来源，AI芯片复杂度提升、存储扩产和国产替代共同拉动高端测试设备需求；合并并删减“半导体测试分选机”重复行。2026-06-16 JPM补充：报告把GPU FT/SLT测试时间延长、TDP提升列为测试设备需求驱动，海外锚为Chroma；长川受益需验证高端SoC/SLT平台订单和AI客户收入，不泛化为所有测试机。</t>
         </is>
       </c>
       <c r="E232" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-16 JPM补充</t>
         </is>
       </c>
     </row>
@@ -7188,17 +7188,17 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>688001</t>
+          <t>688200</t>
         </is>
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>华兴源创</t>
+          <t>华峰测控</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司为工业自动化测试设备与整线系统方案商，产品用于消费电子、半导体集成电路和新能源汽车等；半导体侧包括SiP/芯片测试平台等研发，但AI业绩弹性未单列，合并删减“IC测试板、SiP系统模块测试、半导体测试分选机”重复行。</t>
+          <t>证据中强：2025年报披露公司主营半导体自动化测试系统，收入和利润高增；AI相关弹性主要来自SoC/混合信号等高端测试平台放量与国产替代，现阶段仍以测试设备主业为核心，不单列为AI专用设备。</t>
         </is>
       </c>
       <c r="E233" s="6" t="inlineStr">
@@ -7210,22 +7210,22 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>功率半导体测试设备</t>
+          <t>半导体测试设备</t>
         </is>
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>301369</t>
+          <t>688001</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>联动科技</t>
+          <t>华兴源创</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报显示公司聚焦功率半导体、小信号分立器件测试系统及激光打标设备，并提到紧抓大功率器件、第三代半导体、人工智能产业机遇向SoC测试拓展；AI链条较间接，主板块由泛半导体测试收敛为功率半导体测试设备。</t>
+          <t>证据中：2025年报披露公司为工业自动化测试设备与整线系统方案商，产品用于消费电子、半导体集成电路和新能源汽车等；半导体侧包括SiP/芯片测试平台等研发，但AI业绩弹性未单列，合并删减“IC测试板、SiP系统模块测试、半导体测试分选机”重复行。</t>
         </is>
       </c>
       <c r="E234" s="6" t="inlineStr">
@@ -7237,76 +7237,76 @@
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>AI系统级测试设备</t>
+          <t>功率半导体测试设备</t>
         </is>
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>暂无</t>
+          <t>301369</t>
         </is>
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>暂无成熟A股纯标的（海外锚：致茂电子 2360.TW）</t>
+          <t>联动科技</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>J.P. Morgan Asia Components 2026-06 中文整理版把Chroma的SLT、光通信/CPO、数据中心电源测试标注为三条100%+ CAGR方向；A股映射需拆到长川科技、华峰测控、华兴源创、伟测科技、精智达等子环节逐项验证，当前仅作new_watch，不等同普通半导体测试设备受益。证据B。</t>
+          <t>证据中：2025年报显示公司聚焦功率半导体、小信号分立器件测试系统及激光打标设备，并提到紧抓大功率器件、第三代半导体、人工智能产业机遇向SoC测试拓展；AI链条较间接，主板块由泛半导体测试收敛为功率半导体测试设备。</t>
         </is>
       </c>
       <c r="E235" s="6" t="inlineStr">
         <is>
-          <t>新增；2026-06-16 JPM补充</t>
+          <t>已处理</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>半导体测试探针</t>
+          <t>AI系统级测试设备</t>
         </is>
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>688661</t>
+          <t>暂无</t>
         </is>
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>和林微纳</t>
+          <t>暂无成熟A股纯标的（海外锚：致茂电子 2360.TW）</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报/公开资料显示半导体测试探针业务成为增长引擎，收入同比高增并带动扭亏；公开证据更直接指向测试探针平台，HBM专用探针客户和收入未充分披露，故将“HBM测试探针”降级为半导体测试探针。</t>
+          <t>J.P. Morgan Asia Components 2026-06 中文整理版把Chroma的SLT、光通信/CPO、数据中心电源测试标注为三条100%+ CAGR方向；A股映射需拆到长川科技、华峰测控、华兴源创、伟测科技、精智达等子环节逐项验证，当前仅作new_watch，不等同普通半导体测试设备受益。证据B。</t>
         </is>
       </c>
       <c r="E236" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>新增；2026-06-16 JPM补充</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>晶圆探针台</t>
+          <t>半导体测试探针</t>
         </is>
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>301629</t>
+          <t>688661</t>
         </is>
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>矽电股份</t>
+          <t>和林微纳</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司是中国大陆首家实现12英寸晶圆探针台产业化应用的厂商，产品面向SOC、Memory、CIS、功率器件等测试领域；AI/HBM是行业需求驱动而非已披露专用探针收入，原“HBM测试探针”修正为晶圆探针台。</t>
+          <t>证据中强：2025年报/公开资料显示半导体测试探针业务成为增长引擎，收入同比高增并带动扭亏；公开证据更直接指向测试探针平台，HBM专用探针客户和收入未充分披露，故将“HBM测试探针”降级为半导体测试探针。</t>
         </is>
       </c>
       <c r="E237" s="6" t="inlineStr">
@@ -7318,22 +7318,22 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>半导体测试分选设备</t>
+          <t>晶圆探针台</t>
         </is>
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>603061</t>
+          <t>301629</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>金海通</t>
+          <t>矽电股份</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司专注半导体芯片测试设备，三温测试分选机及大平台超多工位测试分选机需求持续增长、产品销量提升；AI算力芯片和先进封装属于复杂测试应用场景，主板块保留半导体测试分选机。</t>
+          <t>证据强：2025年报披露公司是中国大陆首家实现12英寸晶圆探针台产业化应用的厂商，产品面向SOC、Memory、CIS、功率器件等测试领域；AI/HBM是行业需求驱动而非已披露专用探针收入，原“HBM测试探针”修正为晶圆探针台。</t>
         </is>
       </c>
       <c r="E238" s="6" t="inlineStr">
@@ -7350,17 +7350,17 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>688328</t>
+          <t>603061</t>
         </is>
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>深科达</t>
+          <t>金海通</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报/公告显示公司半导体设备业务增长，转塔式和平移式测试分选机实现批量订单交付，子公司深科达半导体贡献利润；未见TCB热压键合为核心收入，故由TCB修正为半导体测试分选设备。</t>
+          <t>证据强：2025年报披露公司专注半导体芯片测试设备，三温测试分选机及大平台超多工位测试分选机需求持续增长、产品销量提升；AI算力芯片和先进封装属于复杂测试应用场景，主板块保留半导体测试分选机。</t>
         </is>
       </c>
       <c r="E239" s="6" t="inlineStr">
@@ -7372,22 +7372,22 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>半导体检测量测设备</t>
+          <t>半导体测试分选设备</t>
         </is>
       </c>
       <c r="B240" s="3" t="inlineStr">
         <is>
-          <t>688361</t>
+          <t>688328</t>
         </is>
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>中科飞测</t>
+          <t>深科达</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露检测设备和量测设备收入增长，暗场纳米图形晶圆缺陷检测、无图形晶圆缺陷检测、套刻精度量测等产品贡献提升，并拓展电子束/X光技术；先进封装X-Ray作为能力补充并入备注，删除重复行。</t>
+          <t>证据中：2025年报/公告显示公司半导体设备业务增长，转塔式和平移式测试分选机实现批量订单交付，子公司深科达半导体贡献利润；未见TCB热压键合为核心收入，故由TCB修正为半导体测试分选设备。</t>
         </is>
       </c>
       <c r="E240" s="6" t="inlineStr">
@@ -7399,22 +7399,22 @@
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>半导体测试服务</t>
+          <t>半导体检测量测设备</t>
         </is>
       </c>
       <c r="B241" s="3" t="inlineStr">
         <is>
-          <t>688135</t>
+          <t>688361</t>
         </is>
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>利扬芯片</t>
+          <t>中科飞测</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报显示公司主业为集成电路测试方案开发、晶圆测试和成品测试服务，营收创新高且亏损收窄，增长受高算力、存储、汽车电子等芯片测试需求和新客户/新产品导入带动；AI链条为后道测试服务弹性，客户与AI芯片收入未单列。</t>
+          <t>证据强：2025年报披露检测设备和量测设备收入增长，暗场纳米图形晶圆缺陷检测、无图形晶圆缺陷检测、套刻精度量测等产品贡献提升，并拓展电子束/X光技术；先进封装X-Ray作为能力补充并入备注，删除重复行。</t>
         </is>
       </c>
       <c r="E241" s="6" t="inlineStr">
@@ -7431,17 +7431,17 @@
       </c>
       <c r="B242" s="3" t="inlineStr">
         <is>
-          <t>920139</t>
+          <t>688135</t>
         </is>
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>华岭股份</t>
+          <t>利扬芯片</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报显示测试服务仍为核心收入来源，并建设高算力应用芯片开放式测试创新服务平台；但公司2025年亏损扩大，AI/高算力测试仍处研发和客户拓展阶段，主线保留半导体测试服务，备注降级AI兑现强度。</t>
+          <t>证据中强：2025年报显示公司主业为集成电路测试方案开发、晶圆测试和成品测试服务，营收创新高且亏损收窄，增长受高算力、存储、汽车电子等芯片测试需求和新客户/新产品导入带动；AI链条为后道测试服务弹性，客户与AI芯片收入未单列。</t>
         </is>
       </c>
       <c r="E242" s="6" t="inlineStr">
@@ -7458,17 +7458,17 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>688372</t>
+          <t>920139</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>伟测科技</t>
+          <t>华岭股份</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报明确公司聚焦中高端晶圆及成品测试，拓展高算力产品测试，服务CPU/GPU/AI/FPGA、SoC/Chiplet/SiP等测试需求，并披露TSV工艺高性能AI产品整体测试方案研发；主板块由泛半导体测试收敛为高算力芯片测试服务。</t>
+          <t>证据中：2025年报显示测试服务仍为核心收入来源，并建设高算力应用芯片开放式测试创新服务平台；但公司2025年亏损扩大，AI/高算力测试仍处研发和客户拓展阶段，主线保留半导体测试服务，备注降级AI兑现强度。</t>
         </is>
       </c>
       <c r="E243" s="6" t="inlineStr">
@@ -7480,22 +7480,22 @@
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>存储芯片测试设备</t>
+          <t>半导体测试服务</t>
         </is>
       </c>
       <c r="B244" s="3" t="inlineStr">
         <is>
-          <t>688627</t>
+          <t>688372</t>
         </is>
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>精智达</t>
+          <t>伟测科技</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报/公开资料显示半导体存储测试设备业务快速放量，并签订两笔约3.2亿元级半导体重大订单；公司推进高速FT测试机、老化测试修复设备、探针卡及HBM测试设备研发，HBM BI属于未来强化方向，主板块收敛为存储芯片测试设备。</t>
+          <t>证据强：2025年报明确公司聚焦中高端晶圆及成品测试，拓展高算力产品测试，服务CPU/GPU/AI/FPGA、SoC/Chiplet/SiP等测试需求，并披露TSV工艺高性能AI产品整体测试方案研发；主板块由泛半导体测试收敛为高算力芯片测试服务。</t>
         </is>
       </c>
       <c r="E244" s="6" t="inlineStr">
@@ -7507,22 +7507,22 @@
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>半导体洁净室</t>
+          <t>存储芯片测试设备</t>
         </is>
       </c>
       <c r="B245" s="3" t="inlineStr">
         <is>
-          <t>603929</t>
+          <t>688627</t>
         </is>
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>亚翔集成</t>
+          <t>精智达</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司为IC半导体、光电、云计算中心等建厂工程提供洁净室、机电和建筑工程服务，净利润同比高增；AI受益路径来自半导体/存储扩产与厂务资本开支，属于配套基础设施而非芯片产品直接弹性。</t>
+          <t>证据强：2025年报/公开资料显示半导体存储测试设备业务快速放量，并签订两笔约3.2亿元级半导体重大订单；公司推进高速FT测试机、老化测试修复设备、探针卡及HBM测试设备研发，HBM BI属于未来强化方向，主板块收敛为存储芯片测试设备。</t>
         </is>
       </c>
       <c r="E245" s="6" t="inlineStr">
@@ -7539,17 +7539,17 @@
       </c>
       <c r="B246" s="3" t="inlineStr">
         <is>
-          <t>601133</t>
+          <t>603929</t>
         </is>
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>柏诚股份</t>
+          <t>亚翔集成</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报/摘要显示公司主要从事高等级洁净系统集成服务，覆盖半导体及泛半导体、新型显示、生命科学等；2025营收和利润承压且应收/合同资产占比较高，AI链条为晶圆厂扩产配套，保留半导体洁净室但降低弹性强度。</t>
+          <t>证据中强：2025年报披露公司为IC半导体、光电、云计算中心等建厂工程提供洁净室、机电和建筑工程服务，净利润同比高增；AI受益路径来自半导体/存储扩产与厂务资本开支，属于配套基础设施而非芯片产品直接弹性。</t>
         </is>
       </c>
       <c r="E246" s="6" t="inlineStr">
@@ -7566,17 +7566,17 @@
       </c>
       <c r="B247" s="3" t="inlineStr">
         <is>
-          <t>603163</t>
+          <t>601133</t>
         </is>
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>圣晖集成</t>
+          <t>柏诚股份</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报显示公司继续专注洁净室系统集成工程，覆盖设计、采购、施工和维护全链条，主要客户集中在半导体、电子等高科技行业，营收和利润高增；AI受益路径来自晶圆厂/先进封装/存储扩产的厂务资本开支。</t>
+          <t>证据中：2025年报/摘要显示公司主要从事高等级洁净系统集成服务，覆盖半导体及泛半导体、新型显示、生命科学等；2025营收和利润承压且应收/合同资产占比较高，AI链条为晶圆厂扩产配套，保留半导体洁净室但降低弹性强度。</t>
         </is>
       </c>
       <c r="E247" s="6" t="inlineStr">
@@ -7588,22 +7588,22 @@
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>洁净过滤材料</t>
+          <t>半导体洁净室</t>
         </is>
       </c>
       <c r="B248" s="3" t="inlineStr">
         <is>
-          <t>603601</t>
+          <t>603163</t>
         </is>
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>再升科技</t>
+          <t>圣晖集成</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司干净空气材料包括高效空气滤材、PTFE膜等，是FFU、新风系统等核心部件，用于工业电子、生物医药等洁净场景；半导体洁净室链条为间接受益，且2025收入利润承压，故由半导体洁净过滤降级为洁净过滤材料。</t>
+          <t>证据强：2025年报显示公司继续专注洁净室系统集成工程，覆盖设计、采购、施工和维护全链条，主要客户集中在半导体、电子等高科技行业，营收和利润高增；AI受益路径来自晶圆厂/先进封装/存储扩产的厂务资本开支。</t>
         </is>
       </c>
       <c r="E248" s="6" t="inlineStr">
@@ -7615,22 +7615,22 @@
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>半导体洁净过滤</t>
+          <t>洁净过滤材料</t>
         </is>
       </c>
       <c r="B249" s="3" t="inlineStr">
         <is>
-          <t>688376</t>
+          <t>603601</t>
         </is>
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>美埃科技</t>
+          <t>再升科技</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司聚焦工业级超洁净技术，风机过滤单元、过滤器和空气净化设备用于半导体等洁净厂房，并通过收购延伸洁净室墙壁和天花板系统；但2025净利润下滑，半导体项目延期压制业绩弹性。</t>
+          <t>证据中：2025年报披露公司干净空气材料包括高效空气滤材、PTFE膜等，是FFU、新风系统等核心部件，用于工业电子、生物医药等洁净场景；半导体洁净室链条为间接受益，且2025收入利润承压，故由半导体洁净过滤降级为洁净过滤材料。</t>
         </is>
       </c>
       <c r="E249" s="6" t="inlineStr">
@@ -7642,22 +7642,22 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>半导体高纯工艺系统</t>
+          <t>半导体洁净过滤</t>
         </is>
       </c>
       <c r="B250" s="3" t="inlineStr">
         <is>
-          <t>300260</t>
+          <t>688376</t>
         </is>
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>新莱应材</t>
+          <t>美埃科技</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露泛半导体/高纯及超高纯应用材料收入增长，真空和UHP等级管道、管件、阀门、腔体、精密零部件用于半导体制程及厂务；液冷管路属于新布局且规模仍小，合并删减“液冷管路”重复行。</t>
+          <t>证据中强：2025年报披露公司聚焦工业级超洁净技术，风机过滤单元、过滤器和空气净化设备用于半导体等洁净厂房，并通过收购延伸洁净室墙壁和天花板系统；但2025净利润下滑，半导体项目延期压制业绩弹性。</t>
         </is>
       </c>
       <c r="E250" s="6" t="inlineStr">
@@ -7674,17 +7674,17 @@
       </c>
       <c r="B251" s="3" t="inlineStr">
         <is>
-          <t>603690</t>
+          <t>300260</t>
         </is>
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>至纯科技</t>
+          <t>新莱应材</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报摘要披露公司业务围绕高纯工艺系统、制程设备、电子材料、零部件和专业服务，服务晶圆厂建设投产和运营量产；AI链条来自半导体扩产，但2025归母亏损扩大，湿法设备和高纯系统订单修复需继续验证。</t>
+          <t>证据中强：2025年报披露泛半导体/高纯及超高纯应用材料收入增长，真空和UHP等级管道、管件、阀门、腔体、精密零部件用于半导体制程及厂务；液冷管路属于新布局且规模仍小，合并删减“液冷管路”重复行。</t>
         </is>
       </c>
       <c r="E251" s="6" t="inlineStr">
@@ -7701,17 +7701,17 @@
       </c>
       <c r="B252" s="3" t="inlineStr">
         <is>
-          <t>688596</t>
+          <t>603690</t>
         </is>
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>正帆科技</t>
+          <t>至纯科技</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司稳固“制程关键系统、核心工艺材料与零组件、专业服务”三位一体定位，制程关键系统覆盖多数国内一线晶圆厂，GasBox等设备零部件获头部设备厂商采用；合并删减“半导体核心零部件”重复行。</t>
+          <t>证据中：2025年报摘要披露公司业务围绕高纯工艺系统、制程设备、电子材料、零部件和专业服务，服务晶圆厂建设投产和运营量产；AI链条来自半导体扩产，但2025归母亏损扩大，湿法设备和高纯系统订单修复需继续验证。</t>
         </is>
       </c>
       <c r="E252" s="6" t="inlineStr">
@@ -7723,22 +7723,22 @@
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>半导体工艺废气处理</t>
+          <t>半导体高纯工艺系统</t>
         </is>
       </c>
       <c r="B253" s="3" t="inlineStr">
         <is>
-          <t>603324</t>
+          <t>688596</t>
         </is>
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>盛剑环境</t>
+          <t>正帆科技</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
         <is>
-          <t>证据中：公开简称盛剑科技，2025年报显示公司围绕半导体等泛半导体客户提供工艺废气治理、湿电子化学品供应与绿色厂务系统服务；AI受益来自晶圆厂扩产和厂务环保配套，非芯片设备直接弹性。</t>
+          <t>证据中强：2025年报披露公司稳固“制程关键系统、核心工艺材料与零组件、专业服务”三位一体定位，制程关键系统覆盖多数国内一线晶圆厂，GasBox等设备零部件获头部设备厂商采用；合并删减“半导体核心零部件”重复行。</t>
         </is>
       </c>
       <c r="E253" s="6" t="inlineStr">
@@ -7755,17 +7755,17 @@
       </c>
       <c r="B254" s="3" t="inlineStr">
         <is>
-          <t>301030</t>
+          <t>603324</t>
         </is>
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>仕净科技</t>
+          <t>盛剑环境</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>证据弱中：公司有泛半导体/光伏等制程污染防控与废气处理经验，但2025年受光伏客户和资产减值拖累出现大额亏损，半导体AI链条订单和收入证据不足；保留工艺废气处理，但在备注中降级为观察型厂务环保标的。</t>
+          <t>证据中：公开简称盛剑科技，2025年报显示公司围绕半导体等泛半导体客户提供工艺废气治理、湿电子化学品供应与绿色厂务系统服务；AI受益来自晶圆厂扩产和厂务环保配套，非芯片设备直接弹性。</t>
         </is>
       </c>
       <c r="E254" s="6" t="inlineStr">
@@ -7777,22 +7777,22 @@
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>高纯湿电子化学品</t>
+          <t>半导体工艺废气处理</t>
         </is>
       </c>
       <c r="B255" s="3" t="inlineStr">
         <is>
-          <t>688549</t>
+          <t>301030</t>
         </is>
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>中巨芯-U</t>
+          <t>仕净科技</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报显示公司同时覆盖电子湿化学品、电子特种气体和前驱体材料，其中电子湿化学品收入占比约72.5%，电子特气及前驱体占比约23.9%；公司仍亏损，故由ALD-CVD前驱体修正为电子湿化学品。</t>
+          <t>证据弱中：公司有泛半导体/光伏等制程污染防控与废气处理经验，但2025年受光伏客户和资产减值拖累出现大额亏损，半导体AI链条订单和收入证据不足；保留工艺废气处理，但在备注中降级为观察型厂务环保标的。</t>
         </is>
       </c>
       <c r="E255" s="6" t="inlineStr">
@@ -7809,17 +7809,17 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>300655</t>
+          <t>688549</t>
         </is>
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>晶瑞电材</t>
+          <t>中巨芯-U</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报显示公司扭亏并净利润大幅增长，业绩改善主要来自高纯湿化学品量价齐升，光刻胶业务稳健发展且KrF产品已有订单；原半导体光刻胶标签偏窄，收敛为更能解释业绩的高纯湿电子化学品。</t>
+          <t>证据中：2025年报显示公司同时覆盖电子湿化学品、电子特种气体和前驱体材料，其中电子湿化学品收入占比约72.5%，电子特气及前驱体占比约23.9%；公司仍亏损，故由ALD-CVD前驱体修正为电子湿化学品。</t>
         </is>
       </c>
       <c r="E256" s="6" t="inlineStr">
@@ -7831,22 +7831,22 @@
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>光刻胶上游材料</t>
+          <t>高纯湿电子化学品</t>
         </is>
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>300429</t>
+          <t>300655</t>
         </is>
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>强力新材</t>
+          <t>晶瑞电材</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t>公司核心是PCB/LCD/半导体光刻胶光引发剂等电子材料，PSPI先进封装材料项目提供AI先进封装可选弹性；主板块由干膜改为光刻胶上游材料，PSPI并入备注，先进封装电镀液证据不足降级删除。风险是PSPI量产节奏、库存减值、下游竞争和盈利修复。证据B/C。</t>
+          <t>证据中强：2025年报显示公司扭亏并净利润大幅增长，业绩改善主要来自高纯湿化学品量价齐升，光刻胶业务稳健发展且KrF产品已有订单；原半导体光刻胶标签偏窄，收敛为更能解释业绩的高纯湿电子化学品。</t>
         </is>
       </c>
       <c r="E257" s="6" t="inlineStr">
@@ -7858,22 +7858,22 @@
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>半导体光刻胶</t>
+          <t>光刻胶上游材料</t>
         </is>
       </c>
       <c r="B258" s="3" t="inlineStr">
         <is>
-          <t>603650</t>
+          <t>300429</t>
         </is>
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>彤程新材</t>
+          <t>强力新材</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露半导体光刻胶业务高速增长，ArF光刻胶收入实现超800%突破，同时显示光刻胶规模优势稳固；RDL-Bumping属于先进封装光刻材料延伸，合并删减重复行。</t>
+          <t>公司核心是PCB/LCD/半导体光刻胶光引发剂等电子材料，PSPI先进封装材料项目提供AI先进封装可选弹性；主板块由干膜改为光刻胶上游材料，PSPI并入备注，先进封装电镀液证据不足降级删除。风险是PSPI量产节奏、库存减值、下游竞争和盈利修复。证据B/C。</t>
         </is>
       </c>
       <c r="E258" s="6" t="inlineStr">
@@ -7885,22 +7885,22 @@
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>CMP抛光材料</t>
+          <t>半导体光刻胶</t>
         </is>
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>688019</t>
+          <t>603650</t>
         </is>
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>安集科技</t>
+          <t>彤程新材</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司围绕CMP抛光液、功能性湿电子化学品、电镀液及核心原材料形成“3+1”平台，先进封装用TSV、混合键合、聚合物等抛光液在国内客户中作为首选供应商并销售上量；主板块由泛先进封装工艺材料收敛为CMP抛光材料。</t>
+          <t>证据强：2025年报披露半导体光刻胶业务高速增长，ArF光刻胶收入实现超800%突破，同时显示光刻胶规模优势稳固；RDL-Bumping属于先进封装光刻材料延伸，合并删减重复行。</t>
         </is>
       </c>
       <c r="E259" s="6" t="inlineStr">
@@ -7912,22 +7912,22 @@
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>半导体电子特气</t>
+          <t>CMP抛光材料</t>
         </is>
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>688268</t>
+          <t>688019</t>
         </is>
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>华特气体</t>
+          <t>安集科技</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报摘要披露公司特种气体品种数量位居国内前列，已实现57个产品进口替代，覆盖国内8/12英寸集成电路制造厂商超90%客户，并切入全球顶尖半导体供应链；先进封装需求体现在电子特气增量，合并删减泛“先进封装工艺材料”重复行。</t>
+          <t>证据强：2025年报披露公司围绕CMP抛光液、功能性湿电子化学品、电镀液及核心原材料形成“3+1”平台，先进封装用TSV、混合键合、聚合物等抛光液在国内客户中作为首选供应商并销售上量；主板块由泛先进封装工艺材料收敛为CMP抛光材料。</t>
         </is>
       </c>
       <c r="E260" s="6" t="inlineStr">
@@ -7944,22 +7944,22 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>688146</t>
+          <t>688268</t>
         </is>
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>中船特气</t>
+          <t>华特气体</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16 WF6复核后列为“main_candidate / 主受益候选”：公司具备直接WF6合成产能、6N产品能力、较高产能利用率和2027年新增产能规划，AI链条来自3D NAND/HBM/先进逻辑CVD钨沉积需求以及钨出口许可、APT/钨粉、WF6价格链。边界是Kanto Denka/Central Glass“2026-07-01永久停产”未获官方确认，公司也提示未签署新的长期或大额实质性订单，不能把WF6涨价线性外推为业绩。证据A/B/C。</t>
+          <t>证据强：2025年报摘要披露公司特种气体品种数量位居国内前列，已实现57个产品进口替代，覆盖国内8/12英寸集成电路制造厂商超90%客户，并切入全球顶尖半导体供应链；先进封装需求体现在电子特气增量，合并删减泛“先进封装工艺材料”重复行。</t>
         </is>
       </c>
       <c r="E261" s="6" t="inlineStr">
         <is>
-          <t>已处理；2026-06-16复核</t>
+          <t>已处理</t>
         </is>
       </c>
     </row>
@@ -7971,22 +7971,22 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>600378</t>
+          <t>688146</t>
         </is>
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>昊华科技</t>
+          <t>中船特气</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
         <is>
-          <t>证据中强：昊华气体官网披露电子级六氟化钨5N产品，公开互动口径称WF6产能约600吨/年；AI链条来自先进制程/存储芯片CVD钨沉积用电子特气需求，确定性和客户验证透明度弱于中船特气，需跟踪6N升级、客户认证、出口订单和钨粉成本传导。</t>
+          <t>2026-06-16 WF6复核后列为“main_candidate / 主受益候选”：公司具备直接WF6合成产能、6N产品能力、较高产能利用率和2027年新增产能规划，AI链条来自3D NAND/HBM/先进逻辑CVD钨沉积需求以及钨出口许可、APT/钨粉、WF6价格链。边界是Kanto Denka/Central Glass“2026-07-01永久停产”未获官方确认，公司也提示未签署新的长期或大额实质性订单，不能把WF6涨价线性外推为业绩。证据A/B/C。</t>
         </is>
       </c>
       <c r="E262" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已处理；2026-06-16复核</t>
         </is>
       </c>
     </row>
@@ -7998,17 +7998,17 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>688106</t>
+          <t>600378</t>
         </is>
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>金宏气体</t>
+          <t>昊华科技</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露电子特种气体国内市占率约2.81%，电子大宗载气提纯、现场制气及多个半导体/显示项目持续导入；但公司2025年增收不增利、应收较高，主板块由单一电子特气扩为半导体电子气体。</t>
+          <t>证据中强：昊华气体官网披露电子级六氟化钨5N产品，公开互动口径称WF6产能约600吨/年；AI链条来自先进制程/存储芯片CVD钨沉积用电子特气需求，确定性和客户验证透明度弱于中船特气，需跟踪6N升级、客户认证、出口订单和钨粉成本传导。</t>
         </is>
       </c>
       <c r="E263" s="6" t="inlineStr">
@@ -8020,22 +8020,22 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>半导体前驱体材料</t>
+          <t>半导体电子特气</t>
         </is>
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>300346</t>
+          <t>688106</t>
         </is>
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>南大光电</t>
+          <t>金宏气体</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报显示公司围绕先进前驱体、电子特气、光刻胶及配套材料三大核心半导体材料发展，业绩连续增长；光刻胶有产业化突破但收入规模仍需跟踪，主线从光刻胶/ALD-CVD前驱体重复标签收敛为半导体前驱体材料。</t>
+          <t>证据中强：2025年报披露电子特种气体国内市占率约2.81%，电子大宗载气提纯、现场制气及多个半导体/显示项目持续导入；但公司2025年增收不增利、应收较高，主板块由单一电子特气扩为半导体电子气体。</t>
         </is>
       </c>
       <c r="E264" s="6" t="inlineStr">
@@ -8047,22 +8047,22 @@
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>半导体高纯金属靶材</t>
+          <t>半导体前驱体材料</t>
         </is>
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>300666</t>
+          <t>300346</t>
         </is>
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>江丰电子</t>
+          <t>南大光电</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报显示公司核心产品为超高纯金属溅射靶材，覆盖先进制程及存储、逻辑、功率等客户，半导体靶材收入占比高；HBM TSV金属材料属于先进封装/存储升级延伸，证据仍弱于靶材主业，合并删减“HBM TSV金属材料”重复行。</t>
+          <t>证据中强：2025年报显示公司围绕先进前驱体、电子特气、光刻胶及配套材料三大核心半导体材料发展，业绩连续增长；光刻胶有产业化突破但收入规模仍需跟踪，主线从光刻胶/ALD-CVD前驱体重复标签收敛为半导体前驱体材料。</t>
         </is>
       </c>
       <c r="E265" s="6" t="inlineStr">
@@ -8079,17 +8079,17 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>600206</t>
+          <t>300666</t>
         </is>
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>有研新材</t>
+          <t>江丰电子</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司聚焦电子薄膜及贵金属材料等新材料，集成电路及半导体薄膜材料国产化需求持续；高纯金属靶材是更确定主线，HBM TSV金属材料属于先进存储/封装延伸，当前公开证据不足以作为主板块。</t>
+          <t>证据强：2025年报显示公司核心产品为超高纯金属溅射靶材，覆盖先进制程及存储、逻辑、功率等客户，半导体靶材收入占比高；HBM TSV金属材料属于先进封装/存储升级延伸，证据仍弱于靶材主业，合并删减“HBM TSV金属材料”重复行。</t>
         </is>
       </c>
       <c r="E266" s="6" t="inlineStr">
@@ -8101,22 +8101,22 @@
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>半导体先进陶瓷部件</t>
+          <t>半导体高纯金属靶材</t>
         </is>
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>301611</t>
+          <t>600206</t>
         </is>
       </c>
       <c r="C267" s="2" t="inlineStr">
         <is>
-          <t>珂玛科技</t>
+          <t>有研新材</t>
         </is>
       </c>
       <c r="D267" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以半导体先进陶瓷零部件为核心，陶瓷加热器已大批量交付，静电卡盘8/12英寸产品通过客户验证并小规模量产；静电卡盘弹性清晰但收入仍小，主板块由单一静电卡盘修正为半导体先进陶瓷部件。</t>
+          <t>证据中强：2025年报披露公司聚焦电子薄膜及贵金属材料等新材料，集成电路及半导体薄膜材料国产化需求持续；高纯金属靶材是更确定主线，HBM TSV金属材料属于先进存储/封装延伸，当前公开证据不足以作为主板块。</t>
         </is>
       </c>
       <c r="E267" s="6" t="inlineStr">
@@ -8128,22 +8128,22 @@
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>碳化硅衬底</t>
+          <t>半导体先进陶瓷部件</t>
         </is>
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>688234</t>
+          <t>301611</t>
         </is>
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>天岳先进</t>
+          <t>珂玛科技</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司主营碳化硅衬底，导电型SiC衬底全球份额27.6%、8英寸份额51.3%；AI数据中心拉动SiC材料应用是中长期变量，但2025收入下滑并亏损，需跟踪价格和产能利用率。</t>
+          <t>证据中强：2025年报披露公司以半导体先进陶瓷零部件为核心，陶瓷加热器已大批量交付，静电卡盘8/12英寸产品通过客户验证并小规模量产；静电卡盘弹性清晰但收入仍小，主板块由单一静电卡盘修正为半导体先进陶瓷部件。</t>
         </is>
       </c>
       <c r="E268" s="6" t="inlineStr">
@@ -8155,76 +8155,76 @@
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>DRAM存储制造</t>
+          <t>碳化硅衬底</t>
         </is>
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>688825</t>
+          <t>688234</t>
         </is>
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>长鑫科技</t>
+          <t>天岳先进</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
         <is>
-          <t>证据A：DRAM IDM，DDR5已量产并用于服务器，属于AI服务器/数据中心的通用DRAM节点。招股书披露报告期内用于AI算力服务器的DRAM收入占比仍低；不以HBM受益逻辑纳入，HBM量产、客户、订单、收入及独立AI收入均为evidence_absent。来源：上交所招股书（2026-07-22）、公司产品页（2026-09-05复核）。</t>
+          <t>证据强：2025年报披露公司主营碳化硅衬底，导电型SiC衬底全球份额27.6%、8英寸份额51.3%；AI数据中心拉动SiC材料应用是中长期变量，但2025收入下滑并亏损，需跟踪价格和产能利用率。</t>
         </is>
       </c>
       <c r="E269" s="6" t="inlineStr">
         <is>
-          <t>已复核；2026-09-05</t>
+          <t>已处理</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>内存接口芯片</t>
+          <t>DRAM存储制造</t>
         </is>
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>688008</t>
+          <t>688825</t>
         </is>
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>澜起科技</t>
+          <t>长鑫科技</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
         <is>
-          <t>DDR5 RCD/DB、MRCD/MDB、CKD是AI服务器高带宽内存互连核心节点，PCIe Retimer、CXL MXC扩展高速互连第二曲线；主板块收敛为内存接口芯片，HBM、DDR5 SPD、SOCAMM、CXL和CXL内存扩展模组均并入备注或删除，避免误当存储模组/HBM厂商。风险是海外竞争、服务器平台迭代和新品放量节奏。证据A。</t>
+          <t>证据A：DRAM IDM，DDR5已量产并用于服务器，属于AI服务器/数据中心的通用DRAM节点。招股书披露报告期内用于AI算力服务器的DRAM收入占比仍低；不以HBM受益逻辑纳入，HBM量产、客户、订单、收入及独立AI收入均为evidence_absent。来源：上交所招股书（2026-07-22）、公司产品页（2026-09-05复核）。</t>
         </is>
       </c>
       <c r="E270" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>已复核；2026-09-05</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>DDR5 SPD</t>
+          <t>内存接口芯片</t>
         </is>
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>688123</t>
+          <t>688008</t>
         </is>
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>聚辰股份</t>
+          <t>澜起科技</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
         <is>
-          <t>公司具备DDR2/3/4/5内存模组配套SPD、TS等芯片产品，DDR5 SPD受益AI服务器内存模组数量提升，是明确的小芯片弹性节点；主板块保留DDR5 SPD，SOCAMM作为下游内存模组形态并入备注，不单列。风险是DDR5渗透节奏、客户导入、EEPROM周期和价格竞争。证据A。</t>
+          <t>DDR5 RCD/DB、MRCD/MDB、CKD是AI服务器高带宽内存互连核心节点，PCIe Retimer、CXL MXC扩展高速互连第二曲线；主板块收敛为内存接口芯片，HBM、DDR5 SPD、SOCAMM、CXL和CXL内存扩展模组均并入备注或删除，避免误当存储模组/HBM厂商。风险是海外竞争、服务器平台迭代和新品放量节奏。证据A。</t>
         </is>
       </c>
       <c r="E271" s="6" t="inlineStr">
@@ -8236,22 +8236,22 @@
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>高端存储分销</t>
+          <t>DDR5 SPD</t>
         </is>
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>300475</t>
+          <t>688123</t>
         </is>
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>香农芯创</t>
+          <t>聚辰股份</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
         <is>
-          <t>公司以SK海力士核心代理分销为基本盘，向国内云服务器龙头和大型ODM提供存储解决方案；HBM/DDR5紧缺带来强周期弹性，但本质不是HBM制造商。自主海普存储企业级SSD/DRAM开始贡献增量。主板块由HBM改为高端存储分销，风险是存储价格周期、供应商授权、分销毛利和库存。证据A/B。</t>
+          <t>公司具备DDR2/3/4/5内存模组配套SPD、TS等芯片产品，DDR5 SPD受益AI服务器内存模组数量提升，是明确的小芯片弹性节点；主板块保留DDR5 SPD，SOCAMM作为下游内存模组形态并入备注，不单列。风险是DDR5渗透节奏、客户导入、EEPROM周期和价格竞争。证据A。</t>
         </is>
       </c>
       <c r="E272" s="6" t="inlineStr">
@@ -8263,22 +8263,22 @@
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>企业级存储模组</t>
+          <t>高端存储分销</t>
         </is>
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>688525</t>
+          <t>300475</t>
         </is>
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>佰维存储</t>
+          <t>香农芯创</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
         <is>
-          <t>公司企业级存储方案覆盖PCIe/SATA SSD、DDR4/DDR5 RDIMM和CXL内存扩展模组，服务数据中心、服务器和AI工作负载；主板块由DDR5 SPD改为企业级存储模组，SOCAMM、企业级SSD、SSD主控、UFS、晶圆级封测和CXL并入备注或降级。风险是NAND/DRAM价格周期、库存、客户认证和自研控制器/封测兑现。证据B。</t>
+          <t>公司以SK海力士核心代理分销为基本盘，向国内云服务器龙头和大型ODM提供存储解决方案；HBM/DDR5紧缺带来强周期弹性，但本质不是HBM制造商。自主海普存储企业级SSD/DRAM开始贡献增量。主板块由HBM改为高端存储分销，风险是存储价格周期、供应商授权、分销毛利和库存。证据A/B。</t>
         </is>
       </c>
       <c r="E273" s="6" t="inlineStr">
@@ -8295,17 +8295,17 @@
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>301308</t>
+          <t>688525</t>
         </is>
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>江波龙</t>
+          <t>佰维存储</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
         <is>
-          <t>公司企业级eSSD和RDIMM已在互联网、运营商等客户完成验证并批量出货，SOCAMM2、CXL内存扩展、MRDIMM等构成AI服务器存储升级可选项；主板块由SOCAMM改为企业级存储模组，端侧UFS、eMMC、SSD主控、SPU、HLC-iSA、mSSD和CXL并入备注。SOCAMM2仍需收入贡献验证。证据A/B。</t>
+          <t>公司企业级存储方案覆盖PCIe/SATA SSD、DDR4/DDR5 RDIMM和CXL内存扩展模组，服务数据中心、服务器和AI工作负载；主板块由DDR5 SPD改为企业级存储模组，SOCAMM、企业级SSD、SSD主控、UFS、晶圆级封测和CXL并入备注或降级。风险是NAND/DRAM价格周期、库存、客户认证和自研控制器/封测兑现。证据B。</t>
         </is>
       </c>
       <c r="E274" s="6" t="inlineStr">
@@ -8317,22 +8317,22 @@
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>企业级SSD</t>
+          <t>企业级存储模组</t>
         </is>
       </c>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>001309</t>
+          <t>301308</t>
         </is>
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>德明利</t>
+          <t>江波龙</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报摘要披露AI浪潮下公司加快向高容量、高性能固态硬盘拓展，重点聚焦QLC NAND企业级应用方向；自研主控是能力基础，但表格保留最贴近收入承载的“企业级SSD”，删减企业级SSD主控、QLC SSD、AI场景化存储方案重复行。风险是存储价格周期和经营现金流波动。</t>
+          <t>公司企业级eSSD和RDIMM已在互联网、运营商等客户完成验证并批量出货，SOCAMM2、CXL内存扩展、MRDIMM等构成AI服务器存储升级可选项；主板块由SOCAMM改为企业级存储模组，端侧UFS、eMMC、SSD主控、SPU、HLC-iSA、mSSD和CXL并入备注。SOCAMM2仍需收入贡献验证。证据A/B。</t>
         </is>
       </c>
       <c r="E275" s="6" t="inlineStr">
@@ -8344,22 +8344,22 @@
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>企业级SSD主控</t>
+          <t>企业级SSD</t>
         </is>
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>300672</t>
+          <t>001309</t>
         </is>
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>国科微</t>
+          <t>德明利</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
         <is>
-          <t>证据中偏弱：公司固态存储主控芯片实现国产替代，同时布局端侧AI、车载电子、智慧视觉等多条芯片线；AI数据中心企业级SSD客户、收入占比和订单仍未充分披露，保留为SSD主控国产替代观察，基本面需关注2025亏损后毛利修复和研发投入转化。</t>
+          <t>证据中强：2025年报摘要披露AI浪潮下公司加快向高容量、高性能固态硬盘拓展，重点聚焦QLC NAND企业级应用方向；自研主控是能力基础，但表格保留最贴近收入承载的“企业级SSD”，删减企业级SSD主控、QLC SSD、AI场景化存储方案重复行。风险是存储价格周期和经营现金流波动。</t>
         </is>
       </c>
       <c r="E276" s="6" t="inlineStr">
@@ -8376,17 +8376,17 @@
       </c>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>688449</t>
+          <t>300672</t>
         </is>
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>联芸科技</t>
+          <t>国科微</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露SSD主控覆盖SATA、PCIe3.0/4.0/5.0，企业级PCIe Gen5 SSD主控已进入量产测试阶段，并规划PCIe Gen6/Gen7切入数据中心；删减UFS主控重复行，UFS偏终端嵌入式，AI算力弹性以企业级SSD主控为主。</t>
+          <t>证据中偏弱：公司固态存储主控芯片实现国产替代，同时布局端侧AI、车载电子、智慧视觉等多条芯片线；AI数据中心企业级SSD客户、收入占比和订单仍未充分披露，保留为SSD主控国产替代观察，基本面需关注2025亏损后毛利修复和研发投入转化。</t>
         </is>
       </c>
       <c r="E277" s="6" t="inlineStr">
@@ -8398,22 +8398,22 @@
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>AI存储</t>
+          <t>企业级SSD主控</t>
         </is>
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>300302</t>
+          <t>688449</t>
         </is>
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>同有科技</t>
+          <t>联芸科技</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露高端存储在AI智算中心、高性能计算等核心场景推进，NVMe/RDMA高性能分布式文件存储用于智算领域高并发、低延迟需求；主板块保留AI存储，跟踪标杆方案复制、国产化替代和毛利率。</t>
+          <t>证据强：2025年报披露SSD主控覆盖SATA、PCIe3.0/4.0/5.0，企业级PCIe Gen5 SSD主控已进入量产测试阶段，并规划PCIe Gen6/Gen7切入数据中心；删减UFS主控重复行，UFS偏终端嵌入式，AI算力弹性以企业级SSD主控为主。</t>
         </is>
       </c>
       <c r="E278" s="6" t="inlineStr">
@@ -8425,30 +8425,34 @@
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>HBF高带宽闪存</t>
+          <t>AI存储</t>
         </is>
       </c>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>暂无</t>
+          <t>300302</t>
         </is>
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>暂无成熟A股纯标的</t>
+          <t>同有科技</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
         <is>
-          <t>德明利2025半年报提到闪迪HBF结合3D NAND与HBM、适合读取密集型AI推理任务；A股暂无成熟高带宽闪存纯标的。</t>
-        </is>
-      </c>
-      <c r="E279" s="6" t="n"/>
+          <t>证据强：2025年报披露高端存储在AI智算中心、高性能计算等核心场景推进，NVMe/RDMA高性能分布式文件存储用于智算领域高并发、低延迟需求；主板块保留AI存储，跟踪标杆方案复制、国产化替代和毛利率。</t>
+        </is>
+      </c>
+      <c r="E279" s="6" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>Nearline HDD</t>
+          <t>HBF高带宽闪存</t>
         </is>
       </c>
       <c r="B280" s="3" t="inlineStr">
@@ -8463,7 +8467,7 @@
       </c>
       <c r="D280" s="2" t="inlineStr">
         <is>
-          <t>希捷和西部数据官方披露AI数据增长推动数据中心exabyte级低成本存储需求；近线HDD仍主要由海外双寡头主导。</t>
+          <t>德明利2025半年报提到闪迪HBF结合3D NAND与HBM、适合读取密集型AI推理任务；A股暂无成熟高带宽闪存纯标的。</t>
         </is>
       </c>
       <c r="E280" s="6" t="n"/>
@@ -8471,7 +8475,7 @@
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>HAMR-ePMR高容量HDD</t>
+          <t>Nearline HDD</t>
         </is>
       </c>
       <c r="B281" s="3" t="inlineStr">
@@ -8486,7 +8490,7 @@
       </c>
       <c r="D281" s="2" t="inlineStr">
         <is>
-          <t>希捷披露HAMR Mozaic放量，西部数据披露40TB UltraSMR ePMR验证和HAMR 100TB路线；A股暂无成熟HDD主线标的。</t>
+          <t>希捷和西部数据官方披露AI数据增长推动数据中心exabyte级低成本存储需求；近线HDD仍主要由海外双寡头主导。</t>
         </is>
       </c>
       <c r="E281" s="6" t="n"/>
@@ -8494,7 +8498,7 @@
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>高带宽HDD</t>
+          <t>HAMR-ePMR高容量HDD</t>
         </is>
       </c>
       <c r="B282" s="3" t="inlineStr">
@@ -8509,7 +8513,7 @@
       </c>
       <c r="D282" s="2" t="inlineStr">
         <is>
-          <t>西部数据2026 Innovation Day披露High Bandwidth Drive与Dual Pivot提升HDD带宽/IO，服务AI温冷数据层，A股暂无对应纯标的。</t>
+          <t>希捷披露HAMR Mozaic放量，西部数据披露40TB UltraSMR ePMR验证和HAMR 100TB路线；A股暂无成熟HDD主线标的。</t>
         </is>
       </c>
       <c r="E282" s="6" t="n"/>
@@ -8517,7 +8521,7 @@
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>CXL</t>
+          <t>高带宽HDD</t>
         </is>
       </c>
       <c r="B283" s="3" t="inlineStr">
@@ -8532,7 +8536,7 @@
       </c>
       <c r="D283" s="2" t="inlineStr">
         <is>
-          <t>Astera/Broadcom/Marvell主导高速互连芯片，A股除澜起接口芯片外不宜硬凑纯Retimer/PCIe switch标的。</t>
+          <t>西部数据2026 Innovation Day披露High Bandwidth Drive与Dual Pivot提升HDD带宽/IO，服务AI温冷数据层，A股暂无对应纯标的。</t>
         </is>
       </c>
       <c r="E283" s="6" t="n"/>
@@ -8540,22 +8544,22 @@
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>CXL内存扩展模组</t>
+          <t>CXL</t>
         </is>
       </c>
       <c r="B284" s="3" t="inlineStr">
         <is>
+          <t>暂无</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
           <t>暂无成熟A股纯标的</t>
         </is>
       </c>
-      <c r="C284" s="2" t="inlineStr">
-        <is>
-          <t>CXL Switch暂无成熟A股纯标的</t>
-        </is>
-      </c>
       <c r="D284" s="2" t="inlineStr">
         <is>
-          <t>CXL交换/池化控制仍主要由Marvell等海外厂商推进，A股目前缺成熟CXL Switch纯标的。</t>
+          <t>Astera/Broadcom/Marvell主导高速互连芯片，A股除澜起接口芯片外不宜硬凑纯Retimer/PCIe switch标的。</t>
         </is>
       </c>
       <c r="E284" s="6" t="n"/>
@@ -8563,49 +8567,45 @@
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>HBM BI</t>
+          <t>CXL内存扩展模组</t>
         </is>
       </c>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>300567</t>
+          <t>暂无成熟A股纯标的</t>
         </is>
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>精测电子</t>
+          <t>CXL Switch暂无成熟A股纯标的</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
         <is>
-          <t>检测设备平台，2025年报摘要披露推出JH5520 HBM BI测试系统以满足HBM高端存储测试需求，半导体量检测覆盖前道、后道电测和先进封装；主板块改为HBM BI，PCB AOI、半导体量测和先进封装X-Ray并入备注，风险是半导体业务收入占比、客户认证和设备订单兑现。证据A/B。</t>
-        </is>
-      </c>
-      <c r="E285" s="6" t="inlineStr">
-        <is>
-          <t>已处理</t>
-        </is>
-      </c>
+          <t>CXL交换/池化控制仍主要由Marvell等海外厂商推进，A股目前缺成熟CXL Switch纯标的。</t>
+        </is>
+      </c>
+      <c r="E285" s="6" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>AI服务器整机</t>
+          <t>HBM BI</t>
         </is>
       </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>603019</t>
+          <t>300567</t>
         </is>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>中科曙光</t>
+          <t>精测电子</t>
         </is>
       </c>
       <c r="D286" s="2" t="inlineStr">
         <is>
-          <t>证据中强：公司核心是高端计算机、智能计算和算力服务，2025年报披露继续围绕AI算力、液冷散热、高速互联等核心领域投入；AI存储和推理板卡只是配套能力，删减AI存储、AI推理板卡、AI服务器ODM重复行，保留更准确的AI服务器整机/智算底座定位。</t>
+          <t>检测设备平台，2025年报摘要披露推出JH5520 HBM BI测试系统以满足HBM高端存储测试需求，半导体量检测覆盖前道、后道电测和先进封装；主板块改为HBM BI，PCB AOI、半导体量测和先进封装X-Ray并入备注，风险是半导体业务收入占比、客户认证和设备订单兑现。证据A/B。</t>
         </is>
       </c>
       <c r="E286" s="6" t="inlineStr">
@@ -8622,17 +8622,17 @@
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>000977</t>
+          <t>603019</t>
         </is>
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>浪潮信息</t>
+          <t>中科曙光</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露总营收1647.82亿元、同比增长43.25%，主要由服务器产品销售增长驱动；存储交换类收入占比小，删减AI存储重复行，主板块改为AI服务器整机。风险是服务器高增但毛利率偏低，GPU/核心器件供应和价格压力影响利润弹性。</t>
+          <t>证据中强：公司核心是高端计算机、智能计算和算力服务，2025年报披露继续围绕AI算力、液冷散热、高速互联等核心领域投入；AI存储和推理板卡只是配套能力，删减AI存储、AI推理板卡、AI服务器ODM重复行，保留更准确的AI服务器整机/智算底座定位。</t>
         </is>
       </c>
       <c r="E287" s="6" t="inlineStr">
@@ -8649,17 +8649,17 @@
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>000034</t>
+          <t>000977</t>
         </is>
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>神州数码</t>
+          <t>浪潮信息</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露AI相关业务收入330.3亿元、同比增长47.7%，神州鲲泰服务器基于鲲鹏CPU+昇腾NPU支持DeepSeek等大模型私有化部署，并开放国产技术栈AI智算OpenLab；主线是国产算力整机和方案。</t>
+          <t>证据强：2025年报披露总营收1647.82亿元、同比增长43.25%，主要由服务器产品销售增长驱动；存储交换类收入占比小，删减AI存储重复行，主板块改为AI服务器整机。风险是服务器高增但毛利率偏低，GPU/核心器件供应和价格压力影响利润弹性。</t>
         </is>
       </c>
       <c r="E288" s="6" t="inlineStr">
@@ -8676,17 +8676,17 @@
       </c>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>002261</t>
+          <t>000034</t>
         </is>
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>拓维信息</t>
+          <t>神州数码</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报摘要披露公司基于“鲲鹏+昇腾AI”算力底座，推出中心侧高性能服务器、推理服务器和边端终端侧产品；主板块从国产AI服务器收敛为昇腾AI服务器，风险是收入下滑、利润体量仍小。</t>
+          <t>证据中强：2025年报披露AI相关业务收入330.3亿元、同比增长47.7%，神州鲲泰服务器基于鲲鹏CPU+昇腾NPU支持DeepSeek等大模型私有化部署，并开放国产技术栈AI智算OpenLab；主线是国产算力整机和方案。</t>
         </is>
       </c>
       <c r="E289" s="6" t="inlineStr">
@@ -8698,22 +8698,22 @@
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>AI服务器ODM</t>
+          <t>AI服务器整机</t>
         </is>
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>601138</t>
+          <t>002261</t>
         </is>
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>工业富联</t>
+          <t>拓维信息</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司与全球头部客户协同下一代AI服务器及液冷技术，云服务商AI服务器收入同比大增，GPU与ASIC方案产品快速增长；删减“AI服务器机柜”重复行，机柜/液冷作为ODM系统能力纳入备注。</t>
+          <t>证据中：2025年报摘要披露公司基于“鲲鹏+昇腾AI”算力底座，推出中心侧高性能服务器、推理服务器和边端终端侧产品；主板块从国产AI服务器收敛为昇腾AI服务器，风险是收入下滑、利润体量仍小。</t>
         </is>
       </c>
       <c r="E290" s="6" t="inlineStr">
@@ -8730,17 +8730,17 @@
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>603296</t>
+          <t>601138</t>
         </is>
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>华勤技术</t>
+          <t>工业富联</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露华勤数据中心业务形成AI服务器、通用服务器、交换机等全栈产品组合，数据中心业务收入754.75亿元、同比增长51.93%；主板块保留AI服务器ODM，AI PC和终端ODM作为附属受益。</t>
+          <t>证据强：2025年报披露公司与全球头部客户协同下一代AI服务器及液冷技术，云服务商AI服务器收入同比大增，GPU与ASIC方案产品快速增长；删减“AI服务器机柜”重复行，机柜/液冷作为ODM系统能力纳入备注。</t>
         </is>
       </c>
       <c r="E291" s="6" t="inlineStr">
@@ -8752,22 +8752,22 @@
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>算力服务器结构件</t>
+          <t>AI服务器ODM</t>
         </is>
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>002965</t>
+          <t>603296</t>
         </is>
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>祥鑫科技</t>
+          <t>华勤技术</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
         <is>
-          <t>证据中弱：2025年报披露公司在通信设备领域可供应通讯插箱、交换机箱、算力服务器等产品和服务，但汽车业务仍占收入主体且净利润下滑；主板块由AI服务器机柜收敛为算力服务器结构件，AI订单强度需继续验证。</t>
+          <t>证据强：2025年报披露华勤数据中心业务形成AI服务器、通用服务器、交换机等全栈产品组合，数据中心业务收入754.75亿元、同比增长51.93%；主板块保留AI服务器ODM，AI PC和终端ODM作为附属受益。</t>
         </is>
       </c>
       <c r="E292" s="6" t="inlineStr">
@@ -8779,22 +8779,22 @@
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>智能算力产品及服务</t>
+          <t>算力服务器结构件</t>
         </is>
       </c>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>300857</t>
+          <t>002965</t>
         </is>
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>协创数据</t>
+          <t>祥鑫科技</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露智能算力产品及服务收入27.61亿元、同比增长1727.17%、占总收入22.57%，成为第二大收入支柱；原IDC标签不准确，改为智能算力产品及服务。</t>
+          <t>证据中弱：2025年报披露公司在通信设备领域可供应通讯插箱、交换机箱、算力服务器等产品和服务，但汽车业务仍占收入主体且净利润下滑；主板块由AI服务器机柜收敛为算力服务器结构件，AI订单强度需继续验证。</t>
         </is>
       </c>
       <c r="E293" s="6" t="inlineStr">
@@ -8806,22 +8806,22 @@
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>国产AI加速芯片</t>
+          <t>智能算力产品及服务</t>
         </is>
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>688256</t>
+          <t>300857</t>
         </is>
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>寒武纪</t>
+          <t>协创数据</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司云边端智能芯片及板卡矩阵，云端产品线面向服务器和数据中心AI处理，收入大增并首次全年盈利；删减“AI推理板卡”重复行，板卡是产品形态，主板块归入国产AI加速芯片。</t>
+          <t>证据强：2025年报披露智能算力产品及服务收入27.61亿元、同比增长1727.17%、占总收入22.57%，成为第二大收入支柱；原IDC标签不准确，改为智能算力产品及服务。</t>
         </is>
       </c>
       <c r="E294" s="6" t="inlineStr">
@@ -8833,22 +8833,22 @@
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>国产CPU-DCU芯片</t>
+          <t>国产AI加速芯片</t>
         </is>
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>688041</t>
+          <t>688256</t>
         </is>
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>海光信息</t>
+          <t>寒武纪</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报及公开资料显示海光坚持CPU+DCU双芯战略，DCU软件栈适配大模型训练推理并在多行业场景落地；删减“AI推理板卡”重复行，核心价值在国产高端处理器和DCU算力平台。</t>
+          <t>证据强：2025年报披露公司云边端智能芯片及板卡矩阵，云端产品线面向服务器和数据中心AI处理，收入大增并首次全年盈利；删减“AI推理板卡”重复行，板卡是产品形态，主板块归入国产AI加速芯片。</t>
         </is>
       </c>
       <c r="E295" s="6" t="inlineStr">
@@ -8860,22 +8860,22 @@
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>国产GPU芯片</t>
+          <t>国产CPU-DCU芯片</t>
         </is>
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>300474</t>
+          <t>688041</t>
         </is>
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>景嘉微</t>
+          <t>海光信息</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司推进“高性能GPU+边端侧AI SoC芯片”双轮驱动，景宏系列智算模块及整机产品瞄准AI训练和推理；删减“AI推理板卡”重复行，当前仍以国产GPU芯片为主线，亏损和商业化规模是主要风险。</t>
+          <t>证据强：2025年报及公开资料显示海光坚持CPU+DCU双芯战略，DCU软件栈适配大模型训练推理并在多行业场景落地；删减“AI推理板卡”重复行，核心价值在国产高端处理器和DCU算力平台。</t>
         </is>
       </c>
       <c r="E296" s="6" t="inlineStr">
@@ -8887,22 +8887,22 @@
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>AI推理芯片</t>
+          <t>国产GPU芯片</t>
         </is>
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>688343</t>
+          <t>300474</t>
         </is>
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>云天励飞</t>
+          <t>景嘉微</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司构建应用、算法、芯片全栈能力，自研AI推理芯片适配国产大模型、操作系统和推理框架，并推出大模型一体机；一体机为产品化形态，主板块保留AI推理芯片。</t>
+          <t>证据中：2025年报披露公司推进“高性能GPU+边端侧AI SoC芯片”双轮驱动，景宏系列智算模块及整机产品瞄准AI训练和推理；删减“AI推理板卡”重复行，当前仍以国产GPU芯片为主线，亏损和商业化规模是主要风险。</t>
         </is>
       </c>
       <c r="E297" s="6" t="inlineStr">
@@ -8914,22 +8914,22 @@
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>智算网络设备</t>
+          <t>AI推理芯片</t>
         </is>
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>000938</t>
+          <t>688343</t>
         </is>
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>紫光股份</t>
+          <t>云天励飞</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
         <is>
-          <t>证据强：新华三深度覆盖云、网、安、算、存、端，但公司披露中国数据中心交换机份额居前，并在智算网络、800G/CPO交换机和AI算力基础设施上持续推进；删减AI存储、AI服务器ODM重复行，主板块保留最能体现差异化和份额优势的智算交换机。</t>
+          <t>证据中强：2025年报披露公司构建应用、算法、芯片全栈能力，自研AI推理芯片适配国产大模型、操作系统和推理框架，并推出大模型一体机；一体机为产品化形态，主板块保留AI推理芯片。</t>
         </is>
       </c>
       <c r="E298" s="6" t="inlineStr">
@@ -8946,17 +8946,17 @@
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>301165</t>
+          <t>000938</t>
         </is>
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>锐捷网络</t>
+          <t>紫光股份</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露AI智算中心网络方案已服务中国移动、阿里、字节、百度、腾讯等训练/推理大模型场景，数据中心交换机订单加速交付；IDC数据显示中国数据中心交换机市占率第三。</t>
+          <t>证据强：新华三深度覆盖云、网、安、算、存、端，但公司披露中国数据中心交换机份额居前，并在智算网络、800G/CPO交换机和AI算力基础设施上持续推进；删减AI存储、AI服务器ODM重复行，主板块保留最能体现差异化和份额优势的智算交换机。</t>
         </is>
       </c>
       <c r="E299" s="6" t="inlineStr">
@@ -8973,17 +8973,17 @@
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>000063</t>
+          <t>301165</t>
         </is>
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>中兴通讯</t>
+          <t>锐捷网络</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报及公司新闻披露算力业务收入同比约150%，服务器及存储同比超200%，数据中心产品同比增长；公司以自研AI大容量交换芯片支撑智算超节点和万卡级智算中心，主板块从交换机扩展为智算网络设备。</t>
+          <t>证据强：2025年报披露AI智算中心网络方案已服务中国移动、阿里、字节、百度、腾讯等训练/推理大模型场景，数据中心交换机订单加速交付；IDC数据显示中国数据中心交换机市占率第三。</t>
         </is>
       </c>
       <c r="E300" s="6" t="inlineStr">
@@ -8995,22 +8995,22 @@
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>以太网交换芯片</t>
+          <t>智算网络设备</t>
         </is>
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>688702</t>
+          <t>000063</t>
         </is>
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>盛科通信-U</t>
+          <t>中兴通讯</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司主营以太网交换芯片及配套产品，交换芯片收入8.31亿元、占营收72.26%，交换机收入占比较低；删减“智算交换机”重复行，保留最能体现价值量的以太网交换芯片，风险是亏损扩大和高端产品放量节奏。</t>
+          <t>证据强：2025年报及公司新闻披露算力业务收入同比约150%，服务器及存储同比超200%，数据中心产品同比增长；公司以自研AI大容量交换芯片支撑智算超节点和万卡级智算中心，主板块从交换机扩展为智算网络设备。</t>
         </is>
       </c>
       <c r="E301" s="6" t="inlineStr">
@@ -9022,22 +9022,22 @@
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>以太网PHY-交换芯片</t>
+          <t>以太网交换芯片</t>
         </is>
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>688515</t>
+          <t>688702</t>
         </is>
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>裕太微</t>
+          <t>盛科通信-U</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司专注高速有线通信芯片，网通PHY、交换机芯片、网卡芯片已规模量产，网通类产品销量约1.4亿颗，并向数据中心与基站等高价值场景延伸；AI数据中心直接收入仍需跟踪。</t>
+          <t>证据中强：2025年报披露公司主营以太网交换芯片及配套产品，交换芯片收入8.31亿元、占营收72.26%，交换机收入占比较低；删减“智算交换机”重复行，保留最能体现价值量的以太网交换芯片，风险是亏损扩大和高端产品放量节奏。</t>
         </is>
       </c>
       <c r="E302" s="6" t="inlineStr">
@@ -9049,30 +9049,34 @@
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>PCIe Switch</t>
+          <t>以太网PHY-交换芯片</t>
         </is>
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>暂无成熟A股纯标的</t>
+          <t>688515</t>
         </is>
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>暂无成熟A股纯标的</t>
+          <t>裕太微</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr">
         <is>
-          <t>GPU集群内PCIe Switch、NVSwitch和高端交换ASIC主要由NVIDIA、Broadcom、Microchip、Astera等海外厂商主导，A股不硬凑。</t>
-        </is>
-      </c>
-      <c r="E303" s="6" t="n"/>
+          <t>证据中：2025年报披露公司专注高速有线通信芯片，网通PHY、交换机芯片、网卡芯片已规模量产，网通类产品销量约1.4亿颗，并向数据中心与基站等高价值场景延伸；AI数据中心直接收入仍需跟踪。</t>
+        </is>
+      </c>
+      <c r="E303" s="6" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>BMC</t>
+          <t>PCIe Switch</t>
         </is>
       </c>
       <c r="B304" s="3" t="inlineStr">
@@ -9087,7 +9091,7 @@
       </c>
       <c r="D304" s="2" t="inlineStr">
         <is>
-          <t>AI服务器BMC/远程管理芯片以海外和台湾厂商为主，A股目前缺成熟纯标的，先列系统级空白。</t>
+          <t>GPU集群内PCIe Switch、NVSwitch和高端交换ASIC主要由NVIDIA、Broadcom、Microchip、Astera等海外厂商主导，A股不硬凑。</t>
         </is>
       </c>
       <c r="E304" s="6" t="n"/>
@@ -9095,49 +9099,45 @@
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>Edge BMC管理芯片</t>
+          <t>BMC</t>
         </is>
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>688595</t>
+          <t>暂无成熟A股纯标的</t>
         </is>
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>芯海科技</t>
+          <t>暂无成熟A股纯标的</t>
         </is>
       </c>
       <c r="D305" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报摘要披露面向边缘计算及服务器市场的轻量级edge BMC管理芯片已上市并量产销售，同时EC芯片在AI PC量产；保留BMC但改为Edge BMC管理芯片，风险是公司仍亏损且BMC收入规模未单列。</t>
-        </is>
-      </c>
-      <c r="E305" s="6" t="inlineStr">
-        <is>
-          <t>已处理</t>
-        </is>
-      </c>
+          <t>AI服务器BMC/远程管理芯片以海外和台湾厂商为主，A股目前缺成熟纯标的，先列系统级空白。</t>
+        </is>
+      </c>
+      <c r="E305" s="6" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>低抖动时钟源</t>
+          <t>Edge BMC管理芯片</t>
         </is>
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>603738</t>
+          <t>688595</t>
         </is>
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>泰晶科技</t>
+          <t>芯海科技</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报/半年报披露公司开发面向AI数据中心基础设施的312.5MHz差分输出温补振荡器和低抖动可编程振荡器，满足AI数据中心、3.2T光模块、AI算力等需求；主板块保留低抖动时钟源。</t>
+          <t>证据中：2025年报摘要披露面向边缘计算及服务器市场的轻量级edge BMC管理芯片已上市并量产销售，同时EC芯片在AI PC量产；保留BMC但改为Edge BMC管理芯片，风险是公司仍亏损且BMC收入规模未单列。</t>
         </is>
       </c>
       <c r="E306" s="6" t="inlineStr">
@@ -9149,22 +9149,22 @@
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>高频晶振</t>
+          <t>低抖动时钟源</t>
         </is>
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>300460</t>
+          <t>603738</t>
         </is>
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>惠伦晶体</t>
+          <t>泰晶科技</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
         <is>
-          <t>证据弱：2025半年报披露公司主营石英晶体元器件，高频产品和服务器等领域方案商认证具备基础支撑价值；但2025年仍亏损且未见明确AI服务器低抖动订单，主板块由低抖动时钟源降级为高频晶振观察。</t>
+          <t>证据中强：2025年报/半年报披露公司开发面向AI数据中心基础设施的312.5MHz差分输出温补振荡器和低抖动可编程振荡器，满足AI数据中心、3.2T光模块、AI算力等需求；主板块保留低抖动时钟源。</t>
         </is>
       </c>
       <c r="E307" s="6" t="inlineStr">
@@ -9176,22 +9176,22 @@
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>IDC</t>
+          <t>高频晶振</t>
         </is>
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>600845</t>
+          <t>300460</t>
         </is>
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>宝信软件</t>
+          <t>惠伦晶体</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
         <is>
-          <t>工业软件和IDC双主业，宝之云IDC、华北基地、人工智能算力资源池等资产构成算力基础设施运营侧真实映射；DCIM不是公司最核心的AI受益解释。主板块由DCIM改为IDC，原IDC重复行合并删除。风险是钢铁行业软件需求承压、IDC资本开支和上架率、电力成本、AI算力资源池回报周期。证据A/B。</t>
+          <t>证据弱：2025半年报披露公司主营石英晶体元器件，高频产品和服务器等领域方案商认证具备基础支撑价值；但2025年仍亏损且未见明确AI服务器低抖动订单，主板块由低抖动时钟源降级为高频晶振观察。</t>
         </is>
       </c>
       <c r="E308" s="6" t="inlineStr">
@@ -9203,22 +9203,22 @@
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>AIDC智算中心</t>
+          <t>IDC</t>
         </is>
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>300442</t>
+          <t>600845</t>
         </is>
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>润泽科技</t>
+          <t>宝信软件</t>
         </is>
       </c>
       <c r="D309" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报显示AIDC收入25.1亿元、占总收入44.24%，新增交付算力规模220MW且含单体100MW智算中心；合并IDC/算力中心运维，主线改为AIDC智算中心。</t>
+          <t>工业软件和IDC双主业，宝之云IDC、华北基地、人工智能算力资源池等资产构成算力基础设施运营侧真实映射；DCIM不是公司最核心的AI受益解释。主板块由DCIM改为IDC，原IDC重复行合并删除。风险是钢铁行业软件需求承压、IDC资本开支和上架率、电力成本、AI算力资源池回报周期。证据A/B。</t>
         </is>
       </c>
       <c r="E309" s="6" t="inlineStr">
@@ -9230,22 +9230,22 @@
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>IDC及算力租赁</t>
+          <t>AIDC智算中心</t>
         </is>
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>300738</t>
+          <t>300442</t>
         </is>
       </c>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>奥飞数据</t>
+          <t>润泽科技</t>
         </is>
       </c>
       <c r="D310" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露业务为IDC及互联网综合服务，报告期新项目投产并继续推进算力租赁和相关设备销售；AI链受益来自机柜上架和算力需求，保留IDC及算力租赁。</t>
+          <t>证据强：2025年报显示AIDC收入25.1亿元、占总收入44.24%，新增交付算力规模220MW且含单体100MW智算中心；合并IDC/算力中心运维，主线改为AIDC智算中心。</t>
         </is>
       </c>
       <c r="E310" s="6" t="inlineStr">
@@ -9257,22 +9257,22 @@
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>IDC云计算基础设施</t>
+          <t>IDC及算力租赁</t>
         </is>
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>300383</t>
+          <t>300738</t>
         </is>
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>光环新网</t>
+          <t>奥飞数据</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露主营仍是IDC及云计算，AI爆发带动数据中心与云计算需求，并与格灵深瞳合作AI+行业智算云；直接算力运营收入未充分拆分，保留IDC云计算基础设施。</t>
+          <t>证据中：2025年报披露业务为IDC及互联网综合服务，报告期新项目投产并继续推进算力租赁和相关设备销售；AI链受益来自机柜上架和算力需求，保留IDC及算力租赁。</t>
         </is>
       </c>
       <c r="E311" s="6" t="inlineStr">
@@ -9284,22 +9284,22 @@
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>算力中心运维</t>
+          <t>IDC云计算基础设施</t>
         </is>
       </c>
       <c r="B312" s="3" t="inlineStr">
         <is>
-          <t>002929</t>
+          <t>300383</t>
         </is>
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>润建股份</t>
+          <t>光环新网</t>
         </is>
       </c>
       <c r="D312" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露算力网络业务增长、算力中心管理运维和智算云服务推进，但AI及算力收入占比仍较小且归母净利下滑；保留算力中心运维并下调盈利确定性。</t>
+          <t>证据中：2025年报披露主营仍是IDC及云计算，AI爆发带动数据中心与云计算需求，并与格灵深瞳合作AI+行业智算云；直接算力运营收入未充分拆分，保留IDC云计算基础设施。</t>
         </is>
       </c>
       <c r="E312" s="6" t="inlineStr">
@@ -9311,22 +9311,22 @@
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>算力设备交付运维</t>
+          <t>算力中心运维</t>
         </is>
       </c>
       <c r="B313" s="3" t="inlineStr">
         <is>
-          <t>301085</t>
+          <t>002929</t>
         </is>
       </c>
       <c r="C313" s="2" t="inlineStr">
         <is>
-          <t>亚康股份</t>
+          <t>润建股份</t>
         </is>
       </c>
       <c r="D313" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报摘要披露向富士康、英业达、华勤、浪潮等算力服务器制造商提供交付及售后维保，并从传统数据中心向AI智算中心运维升级；公司亏损，主线为算力设备交付运维。</t>
+          <t>证据中：2025年报披露算力网络业务增长、算力中心管理运维和智算云服务推进，但AI及算力收入占比仍较小且归母净利下滑；保留算力中心运维并下调盈利确定性。</t>
         </is>
       </c>
       <c r="E313" s="6" t="inlineStr">
@@ -9338,22 +9338,22 @@
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>AI智能终端ODM</t>
+          <t>算力设备交付运维</t>
         </is>
       </c>
       <c r="B314" s="3" t="inlineStr">
         <is>
-          <t>603341</t>
+          <t>301085</t>
         </is>
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>龙旗科技</t>
+          <t>亚康股份</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露AI PC实现全平台产品设计与量产落地并获得全球头部客户订单，智能眼镜实现多场景、多品类规模化量产，AIoT业务覆盖智能手表/手环和智能眼镜；主板块从智能终端ODM细化为AI智能终端ODM。风险是手机/平板仍占大盘，新业务弹性需看AI PC、智能眼镜收入占比和毛利。</t>
+          <t>证据中：2025年报摘要披露向富士康、英业达、华勤、浪潮等算力服务器制造商提供交付及售后维保，并从传统数据中心向AI智算中心运维升级；公司亏损，主线为算力设备交付运维。</t>
         </is>
       </c>
       <c r="E314" s="6" t="inlineStr">
@@ -9365,27 +9365,27 @@
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>端侧AI SoC</t>
+          <t>AI智能终端ODM</t>
         </is>
       </c>
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>603893</t>
+          <t>603341</t>
         </is>
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>瑞芯微</t>
+          <t>龙旗科技</t>
         </is>
       </c>
       <c r="D315" s="2" t="inlineStr">
         <is>
-          <t>证据强：2026年一季报及2026年半年度业绩预告显示，公司采用“AIoT SoC算力平台+AI协处理器”双轨路线，RK3588、RK3576、RV11系列持续高速增长，RK182X已量产并预计下半年开始放量；以RK3588为例，芯片集成CPU、GPU、6TOPS自研NPU、ISP及8K音视频编解码能力，终端覆盖机器人、机器视觉/安防、工业控制、智能座舱、商显/办公、智能家居及教育娱乐等消费电子。2026H1预告营收28.70—29.10亿元、归母净利润8.50—9.10亿元、扣非净利润8.30—8.90亿元（均未经审计）。主板块归入端侧AI SoC；风险是存储及载板等原材料涨价/短缺、消费类终端承压，以及新品导入和放量不及预期。</t>
+          <t>证据中强：2025年报披露AI PC实现全平台产品设计与量产落地并获得全球头部客户订单，智能眼镜实现多场景、多品类规模化量产，AIoT业务覆盖智能手表/手环和智能眼镜；主板块从智能终端ODM细化为AI智能终端ODM。风险是手机/平板仍占大盘，新业务弹性需看AI PC、智能眼镜收入占比和毛利。</t>
         </is>
       </c>
       <c r="E315" s="6" t="inlineStr">
         <is>
-          <t>更新；2026-07-25</t>
+          <t>已处理</t>
         </is>
       </c>
     </row>
@@ -9397,22 +9397,22 @@
       </c>
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>300458</t>
+          <t>603893</t>
         </is>
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>全志科技</t>
+          <t>瑞芯微</t>
         </is>
       </c>
       <c r="D316" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司实现CPU、GPU、NPU、DSP及RISC-V协处理器复杂异构芯片规模化量产，智能终端应用处理器是核心业务；删减AI眼镜应用处理器重复行，AI眼镜只是下游应用之一，主板块保留端侧AI SoC。</t>
+          <t>证据强：2026年一季报及2026年半年度业绩预告显示，公司采用“AIoT SoC算力平台+AI协处理器”双轨路线，RK3588、RK3576、RV11系列持续高速增长，RK182X已量产并预计下半年开始放量；以RK3588为例，芯片集成CPU、GPU、6TOPS自研NPU、ISP及8K音视频编解码能力，终端覆盖机器人、机器视觉/安防、工业控制、智能座舱、商显/办公、智能家居及教育娱乐等消费电子。2026H1预告营收28.70—29.10亿元、归母净利润8.50—9.10亿元、扣非净利润8.30—8.90亿元（均未经审计）。主板块归入端侧AI SoC；风险是存储及载板等原材料涨价/短缺、消费类终端承压，以及新品导入和放量不及预期。</t>
         </is>
       </c>
       <c r="E316" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>更新；2026-07-25</t>
         </is>
       </c>
     </row>
@@ -9424,17 +9424,17 @@
       </c>
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>688099</t>
+          <t>300458</t>
         </is>
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>晶晨股份</t>
+          <t>全志科技</t>
         </is>
       </c>
       <c r="D317" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露智能多媒体及显示SoC仍是核心收入来源，AIoT SoC收入16.40亿元、同比增长8.50%，AIoT SoC集成NPU、DSP、视觉处理单元、ISP及编解码器并获Google EDLA认证；主板块从端侧AIoT SoC收敛为端侧AI SoC，跟踪端侧大模型适配、头部客户新品和经营现金流修复。</t>
+          <t>证据中强：2025年报披露公司实现CPU、GPU、NPU、DSP及RISC-V协处理器复杂异构芯片规模化量产，智能终端应用处理器是核心业务；删减AI眼镜应用处理器重复行，AI眼镜只是下游应用之一，主板块保留端侧AI SoC。</t>
         </is>
       </c>
       <c r="E317" s="6" t="inlineStr">
@@ -9451,71 +9451,71 @@
       </c>
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>301536</t>
+          <t>688099</t>
         </is>
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
-          <t>星宸科技</t>
+          <t>晶晨股份</t>
         </is>
       </c>
       <c r="D318" s="2" t="inlineStr">
         <is>
-          <t>证据强（截至2026-07-25）：公司以视觉AI SoC为核心，核心芯片集成ISP、NPU、编解码、音频/显示等IP；主要产品/目标终端包括IPC/NVR（SSR670G）、家用服务及户外等机器人、智能家居/办公/工业、智能穿戴和车载记录仪/DMS/OMS/CMS/L0-L2辅助驾驶，另布局SPAD 3D感知与蓝牙。已形成收入：2025年智能安防19.35亿元/65.10%、智能物联6.58亿元/22.14%、智能车载3.18亿元/10.69%；2026H1预告收入26.2—27.2亿元、归母8.2—9.0亿元、扣非7.0—7.8亿元（未经审计；7月22日公告称无需修正），SSR670系列公司称已大规模商用。商业化边界：AI眼镜SSC309QL仅小规模量产，另有5—6家客户开发中，订单/独立收入N/A；机器人2025年出货超1,000万颗但独立收入N/A，具身“小脑/大脑”仍在研；SS901公司IR称已在国内一线自主品牌主力车型量产上车，其他车载/3D项目的导入或规划不等于订单/收入。PE(TTM，用户口径)=24.4—28.4x：总市值555.82亿元（东方财富，2026-07-24收盘）÷[(2026H1扣非预告7.0—7.8亿元−2026Q1扣非2.0998亿元)×4]，非标准近四季PE。证据状态：财务/分部=confirmed_official；产品/客户进展=company_claim；估值=market_data_vendor；annualized_core_gap_status=insufficient、formal_surprise_status=N/A（缺公告前FY归母点时共识）。风险：半年度预告待8月27日正式半年报验证，毛利率、现金流、存货、价量与新品放量持续性待核。</t>
+          <t>证据中强：2025年报披露智能多媒体及显示SoC仍是核心收入来源，AIoT SoC收入16.40亿元、同比增长8.50%，AIoT SoC集成NPU、DSP、视觉处理单元、ISP及编解码器并获Google EDLA认证；主板块从端侧AIoT SoC收敛为端侧AI SoC，跟踪端侧大模型适配、头部客户新品和经营现金流修复。</t>
         </is>
       </c>
       <c r="E318" s="6" t="inlineStr">
         <is>
-          <t>更新；2026-07-25</t>
+          <t>已处理</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜主控SoC</t>
+          <t>端侧AI SoC</t>
         </is>
       </c>
       <c r="B319" s="3" t="inlineStr">
         <is>
-          <t>688608</t>
+          <t>301536</t>
         </is>
       </c>
       <c r="C319" s="2" t="inlineStr">
         <is>
-          <t>恒玄科技</t>
+          <t>星宸科技</t>
         </is>
       </c>
       <c r="D319" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司主营低功耗无线计算SoC，芯片集成CPU、嵌入式NPU、ISP、DSP、蓝牙/Wi-Fi等模块；BES6100面向智能眼镜等低功耗终端，6nm工艺，集成多核Cortex-A、NPU、GPU，可运行Linux/Android并支持端侧AI推理。风险是AI眼镜SoC仍处放量早期，需跟踪客户导入和量产节奏。</t>
+          <t>证据强（截至2026-07-25）：公司以视觉AI SoC为核心，核心芯片集成ISP、NPU、编解码、音频/显示等IP；主要产品/目标终端包括IPC/NVR（SSR670G）、家用服务及户外等机器人、智能家居/办公/工业、智能穿戴和车载记录仪/DMS/OMS/CMS/L0-L2辅助驾驶，另布局SPAD 3D感知与蓝牙。已形成收入：2025年智能安防19.35亿元/65.10%、智能物联6.58亿元/22.14%、智能车载3.18亿元/10.69%；2026H1预告收入26.2—27.2亿元、归母8.2—9.0亿元、扣非7.0—7.8亿元（未经审计；7月22日公告称无需修正），SSR670系列公司称已大规模商用。商业化边界：AI眼镜SSC309QL仅小规模量产，另有5—6家客户开发中，订单/独立收入N/A；机器人2025年出货超1,000万颗但独立收入N/A，具身“小脑/大脑”仍在研；SS901公司IR称已在国内一线自主品牌主力车型量产上车，其他车载/3D项目的导入或规划不等于订单/收入。PE(TTM，用户口径)=24.4—28.4x：总市值555.82亿元（东方财富，2026-07-24收盘）÷[(2026H1扣非预告7.0—7.8亿元−2026Q1扣非2.0998亿元)×4]，非标准近四季PE。证据状态：财务/分部=confirmed_official；产品/客户进展=company_claim；估值=market_data_vendor；annualized_core_gap_status=insufficient、formal_surprise_status=N/A（缺公告前FY归母点时共识）。风险：半年度预告待8月27日正式半年报验证，毛利率、现金流、存货、价量与新品放量持续性待核。</t>
         </is>
       </c>
       <c r="E319" s="6" t="inlineStr">
         <is>
-          <t>已处理</t>
+          <t>更新；2026-07-25</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>智能穿戴SoC</t>
+          <t>AI眼镜主控SoC</t>
         </is>
       </c>
       <c r="B320" s="3" t="inlineStr">
         <is>
-          <t>688049</t>
+          <t>688608</t>
         </is>
       </c>
       <c r="C320" s="2" t="inlineStr">
         <is>
-          <t>炬芯科技</t>
+          <t>恒玄科技</t>
         </is>
       </c>
       <c r="D320" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报摘要披露公司构建低功耗大算力芯片硬件架构、端侧AI开发工具和存内计算CIM，CPU+DSP+NPU架构提升端侧AI能效；智能穿戴SoC覆盖手表/手环、AI眼镜等，主板块保留智能穿戴SoC，AI眼镜属于穿戴场景扩展而非单独主线。</t>
+          <t>证据强：2025年报披露公司主营低功耗无线计算SoC，芯片集成CPU、嵌入式NPU、ISP、DSP、蓝牙/Wi-Fi等模块；BES6100面向智能眼镜等低功耗终端，6nm工艺，集成多核Cortex-A、NPU、GPU，可运行Linux/Android并支持端侧AI推理。风险是AI眼镜SoC仍处放量早期，需跟踪客户导入和量产节奏。</t>
         </is>
       </c>
       <c r="E320" s="6" t="inlineStr">
@@ -9527,22 +9527,22 @@
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>端侧音视频SoC</t>
+          <t>智能穿戴SoC</t>
         </is>
       </c>
       <c r="B321" s="3" t="inlineStr">
         <is>
-          <t>688332</t>
+          <t>688049</t>
         </is>
       </c>
       <c r="C321" s="2" t="inlineStr">
         <is>
-          <t>中科蓝讯</t>
+          <t>炬芯科技</t>
         </is>
       </c>
       <c r="D321" s="2" t="inlineStr">
         <is>
-          <t>证据中：公司专注低功耗无线音频SoC，2025年报披露形成蓝牙耳机、智能穿戴、AIoT、AI语音识别、Wi-Fi、视频芯片等产品线，并向AI玩具、AI眼镜、AI音箱扩展；主板块保留端侧音视频SoC。风险是2025净利高增主要受投资公允价值影响，扣非和主业毛利需单独跟踪。</t>
+          <t>证据中强：2025年报摘要披露公司构建低功耗大算力芯片硬件架构、端侧AI开发工具和存内计算CIM，CPU+DSP+NPU架构提升端侧AI能效；智能穿戴SoC覆盖手表/手环、AI眼镜等，主板块保留智能穿戴SoC，AI眼镜属于穿戴场景扩展而非单独主线。</t>
         </is>
       </c>
       <c r="E321" s="6" t="inlineStr">
@@ -9554,22 +9554,22 @@
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>端侧AI MCU</t>
+          <t>端侧音视频SoC</t>
         </is>
       </c>
       <c r="B322" s="3" t="inlineStr">
         <is>
-          <t>688018</t>
+          <t>688332</t>
         </is>
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>乐鑫科技</t>
+          <t>中科蓝讯</t>
         </is>
       </c>
       <c r="D322" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以AIoT为核心，芯片、模组和开发套件保持增长；官方ESP32-P4为双核RISC-V高性能MCU，具备AI指令扩展、先进内存子系统和高速外设，面向HMI、边缘计算、视觉AI等嵌入式场景。风险是AI算力较SoC/NPU平台更轻量，需跟踪高端新品放量和客户结构。</t>
+          <t>证据中：公司专注低功耗无线音频SoC，2025年报披露形成蓝牙耳机、智能穿戴、AIoT、AI语音识别、Wi-Fi、视频芯片等产品线，并向AI玩具、AI眼镜、AI音箱扩展；主板块保留端侧音视频SoC。风险是2025净利高增主要受投资公允价值影响，扣非和主业毛利需单独跟踪。</t>
         </is>
       </c>
       <c r="E322" s="6" t="inlineStr">
@@ -9581,22 +9581,22 @@
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>端侧AI蜂窝模组</t>
+          <t>端侧AI MCU</t>
         </is>
       </c>
       <c r="B323" s="3" t="inlineStr">
         <is>
-          <t>603236</t>
+          <t>688018</t>
         </is>
       </c>
       <c r="C323" s="2" t="inlineStr">
         <is>
-          <t>移远通信</t>
+          <t>乐鑫科技</t>
         </is>
       </c>
       <c r="D323" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露物联网需求回暖，边缘计算、混合现实、大模型与物联网融合加速；公司推出支持主流AI大模型端侧部署的5G智能座舱模组，并依托智能模组、AI大模型、主控板、算力卡和自研算法打造多层级端侧AI方案。主板块保留端侧AI蜂窝模组，跟踪AI模组收入占比和毛利提升。</t>
+          <t>证据中强：2025年报披露公司以AIoT为核心，芯片、模组和开发套件保持增长；官方ESP32-P4为双核RISC-V高性能MCU，具备AI指令扩展、先进内存子系统和高速外设，面向HMI、边缘计算、视觉AI等嵌入式场景。风险是AI算力较SoC/NPU平台更轻量，需跟踪高端新品放量和客户结构。</t>
         </is>
       </c>
       <c r="E323" s="6" t="inlineStr">
@@ -9608,22 +9608,22 @@
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>高算力智能模组</t>
+          <t>端侧AI蜂窝模组</t>
         </is>
       </c>
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>002881</t>
+          <t>603236</t>
         </is>
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>美格智能</t>
+          <t>移远通信</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露无线通信模组正向智能模组、高算力模组升级，公司的智能模组和高算力模组是物联网终端侧、边缘侧计算能力承载平台，并推动端侧AI在物联网领域落地；主板块从端侧AI蜂窝模组细化为高算力智能模组，跟踪海外收入、车载/AR/VR等大颗粒市场和毛利修复。</t>
+          <t>证据强：2025年报披露物联网需求回暖，边缘计算、混合现实、大模型与物联网融合加速；公司推出支持主流AI大模型端侧部署的5G智能座舱模组，并依托智能模组、AI大模型、主控板、算力卡和自研算法打造多层级端侧AI方案。主板块保留端侧AI蜂窝模组，跟踪AI模组收入占比和毛利提升。</t>
         </is>
       </c>
       <c r="E324" s="6" t="inlineStr">
@@ -9635,22 +9635,22 @@
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>端侧AI模组</t>
+          <t>高算力智能模组</t>
         </is>
       </c>
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>300638</t>
+          <t>002881</t>
         </is>
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>广和通</t>
+          <t>美格智能</t>
         </is>
       </c>
       <c r="D325" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司发布Fibocom AI Stack端侧AI解决方案及覆盖1T-50T算力的“星云”AI模组矩阵，支持不同参数端侧大模型部署，应用于AI玩具、机器人等终端；主板块保留端侧AI模组，跟踪星云系列出货、AI解决方案收入占比和客户落地。</t>
+          <t>证据中强：2025年报披露无线通信模组正向智能模组、高算力模组升级，公司的智能模组和高算力模组是物联网终端侧、边缘侧计算能力承载平台，并推动端侧AI在物联网领域落地；主板块从端侧AI蜂窝模组细化为高算力智能模组，跟踪海外收入、车载/AR/VR等大颗粒市场和毛利修复。</t>
         </is>
       </c>
       <c r="E325" s="6" t="inlineStr">
@@ -9662,22 +9662,22 @@
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>AIOS端侧智能</t>
+          <t>端侧AI模组</t>
         </is>
       </c>
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>300496</t>
+          <t>300638</t>
         </is>
       </c>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>中科创达</t>
+          <t>广和通</t>
         </is>
       </c>
       <c r="D326" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司以AIOS为核心战略，覆盖端云协同、AI智能体和行业AI，并在智能汽车、AI眼镜、机器人等端侧场景落地；主板块由端侧智能OS升级为AIOS端侧智能。</t>
+          <t>证据强：2025年报披露公司发布Fibocom AI Stack端侧AI解决方案及覆盖1T-50T算力的“星云”AI模组矩阵，支持不同参数端侧大模型部署，应用于AI玩具、机器人等终端；主板块保留端侧AI模组，跟踪星云系列出货、AI解决方案收入占比和客户落地。</t>
         </is>
       </c>
       <c r="E326" s="6" t="inlineStr">
@@ -9689,22 +9689,22 @@
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>AR光波导</t>
+          <t>AIOS端侧智能</t>
         </is>
       </c>
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>002273</t>
+          <t>300496</t>
         </is>
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>水晶光电</t>
+          <t>中科创达</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
         <is>
-          <t>精密镀膜、微纳光学和光电封测能力较强，AR/VR领域反射光波导及核心光学元件为公司重点工程，AI眼镜是更直接的未来映射；主板块改为AR光波导，微透镜并入备注，CPO硅透镜研发仅作远期观察，风险是AR大客户量产节奏、消费电子大客户依赖和光通信收入兑现。证据B。</t>
+          <t>证据强：2025年报披露公司以AIOS为核心战略，覆盖端云协同、AI智能体和行业AI，并在智能汽车、AI眼镜、机器人等端侧场景落地；主板块由端侧智能OS升级为AIOS端侧智能。</t>
         </is>
       </c>
       <c r="E327" s="6" t="inlineStr">
@@ -9716,22 +9716,22 @@
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜光学模组</t>
+          <t>AR光波导</t>
         </is>
       </c>
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>300433</t>
+          <t>002273</t>
         </is>
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>蓝思科技</t>
+          <t>水晶光电</t>
         </is>
       </c>
       <c r="D328" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司是AI硬件全产业链一站式精密制造解决方案提供商，AI眼镜领域具备材料、光学、结构件到整机组装全栈能力，已实现国内头部客户整机组装和海外头部客户精密零组件规模化交付，并在光波导镜片高精度自动化组装等领域突破；主板块从AI眼镜光波导扩展为AI眼镜光学模组。</t>
+          <t>精密镀膜、微纳光学和光电封测能力较强，AR/VR领域反射光波导及核心光学元件为公司重点工程，AI眼镜是更直接的未来映射；主板块改为AR光波导，微透镜并入备注，CPO硅透镜研发仅作远期观察，风险是AR大客户量产节奏、消费电子大客户依赖和光通信收入兑现。证据B。</t>
         </is>
       </c>
       <c r="E328" s="6" t="inlineStr">
@@ -9743,22 +9743,22 @@
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>AR投影光机</t>
+          <t>AI眼镜光学模组</t>
         </is>
       </c>
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>688010</t>
+          <t>300433</t>
         </is>
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>福光股份</t>
+          <t>蓝思科技</t>
         </is>
       </c>
       <c r="D329" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司主营特种及民用光学镜头、光电系统和光学元组件，研发项目中M003 MicroLED AR显示模组处于产业化推广，应用于AR领域；投影光机可用于AR/可穿戴设备。主板块保留AR投影光机，但AI眼镜收入纯度和客户放量仍需继续验证，扣非盈利仍承压。</t>
+          <t>证据强：2025年报披露公司是AI硬件全产业链一站式精密制造解决方案提供商，AI眼镜领域具备材料、光学、结构件到整机组装全栈能力，已实现国内头部客户整机组装和海外头部客户精密零组件规模化交付，并在光波导镜片高精度自动化组装等领域突破；主板块从AI眼镜光波导扩展为AI眼镜光学模组。</t>
         </is>
       </c>
       <c r="E329" s="6" t="inlineStr">
@@ -9770,22 +9770,22 @@
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>硅基OLED微显示</t>
+          <t>AR投影光机</t>
         </is>
       </c>
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>688496</t>
+          <t>688010</t>
         </is>
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>清越科技</t>
+          <t>福光股份</t>
         </is>
       </c>
       <c r="D330" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司形成PMOLED、电子纸模组与硅基OLED微显示器三大业务，硅基OLED用于AR智能眼镜、VR头显等近眼显示；Micro-OLED高亮高效结构器件等项目继续推进。主板块保留硅基OLED微显示，但公司2025亏损扩大，需跟踪硅基OLED量产客户和盈利拐点。</t>
+          <t>证据中：2025年报披露公司主营特种及民用光学镜头、光电系统和光学元组件，研发项目中M003 MicroLED AR显示模组处于产业化推广，应用于AR领域；投影光机可用于AR/可穿戴设备。主板块保留AR投影光机，但AI眼镜收入纯度和客户放量仍需继续验证，扣非盈利仍承压。</t>
         </is>
       </c>
       <c r="E330" s="6" t="inlineStr">
@@ -9797,22 +9797,22 @@
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜MicroLED光机</t>
+          <t>硅基OLED微显示</t>
         </is>
       </c>
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>300296</t>
+          <t>688496</t>
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>利亚德</t>
+          <t>清越科技</t>
         </is>
       </c>
       <c r="D331" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年度总经理工作报告披露公司已推出基于MicroLED光机的AR眼镜，并发布AI玩具等大众消费AI创新产品；MicroLED仍是新战略周期重点增长方向。主板块保留AI眼镜MicroLED光机，风险是公司收入主体仍为LED显示和文旅，AI眼镜商业化仍早期。</t>
+          <t>证据中：2025年报披露公司形成PMOLED、电子纸模组与硅基OLED微显示器三大业务，硅基OLED用于AR智能眼镜、VR头显等近眼显示；Micro-OLED高亮高效结构器件等项目继续推进。主板块保留硅基OLED微显示，但公司2025亏损扩大，需跟踪硅基OLED量产客户和盈利拐点。</t>
         </is>
       </c>
       <c r="E331" s="6" t="inlineStr">
@@ -9824,22 +9824,22 @@
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜MicroLED微显示</t>
+          <t>AI眼镜MicroLED光机</t>
         </is>
       </c>
       <c r="B332" s="3" t="inlineStr">
         <is>
-          <t>300323</t>
+          <t>300296</t>
         </is>
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>京东方华灿</t>
+          <t>利亚德</t>
         </is>
       </c>
       <c r="D332" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025投资者关系记录披露MicroLED技术可用于具备显示功能的AI眼镜，公司配合不同客户需求提供解决方案并提升性能与良率；2025年报披露MicroLED技术研发及产业化项目推进高亮度、高对比度、高色彩饱和度芯片。主板块保留AI眼镜MicroLED微显示，风险是公司仍亏损，产业化和客户放量需跟踪。</t>
+          <t>证据中强：2025年度总经理工作报告披露公司已推出基于MicroLED光机的AR眼镜，并发布AI玩具等大众消费AI创新产品；MicroLED仍是新战略周期重点增长方向。主板块保留AI眼镜MicroLED光机，风险是公司收入主体仍为LED显示和文旅，AI眼镜商业化仍早期。</t>
         </is>
       </c>
       <c r="E332" s="6" t="inlineStr">
@@ -9851,22 +9851,22 @@
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>MicroLED芯片</t>
+          <t>AI眼镜MicroLED微显示</t>
         </is>
       </c>
       <c r="B333" s="3" t="inlineStr">
         <is>
-          <t>600703</t>
+          <t>300323</t>
         </is>
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>三安光电</t>
+          <t>京东方华灿</t>
         </is>
       </c>
       <c r="D333" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露Mini/Micro LED高端产品占比提升，Micro LED芯片在中大型显示增长，并切入AR眼镜、AI数据中心光互连等应用；删减“化合物半导体”重复行，SiC/GaN等平台能力在备注降级说明。</t>
+          <t>证据中：2025投资者关系记录披露MicroLED技术可用于具备显示功能的AI眼镜，公司配合不同客户需求提供解决方案并提升性能与良率；2025年报披露MicroLED技术研发及产业化项目推进高亮度、高对比度、高色彩饱和度芯片。主板块保留AI眼镜MicroLED微显示，风险是公司仍亏损，产业化和客户放量需跟踪。</t>
         </is>
       </c>
       <c r="E333" s="6" t="inlineStr">
@@ -9878,22 +9878,22 @@
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>OLED-MicroLED显示</t>
+          <t>MicroLED芯片</t>
         </is>
       </c>
       <c r="B334" s="3" t="inlineStr">
         <is>
-          <t>002387</t>
+          <t>600703</t>
         </is>
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>维信诺</t>
+          <t>三安光电</t>
         </is>
       </c>
       <c r="D334" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露维信诺围绕AI新场景推进智能终端、智能影像、智慧家居等显示供货，并持续推进ViP、Micro-LED等显示技术；真实受益节点是AI终端显示，MicroLED更多体现技术储备和参股生态。</t>
+          <t>证据中强：2025年报披露Mini/Micro LED高端产品占比提升，Micro LED芯片在中大型显示增长，并切入AR眼镜、AI数据中心光互连等应用；删减“化合物半导体”重复行，SiC/GaN等平台能力在备注降级说明。</t>
         </is>
       </c>
       <c r="E334" s="6" t="inlineStr">
@@ -9905,22 +9905,22 @@
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜CIS</t>
+          <t>OLED-MicroLED显示</t>
         </is>
       </c>
       <c r="B335" s="3" t="inlineStr">
         <is>
-          <t>688213</t>
+          <t>002387</t>
         </is>
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>思特威</t>
+          <t>维信诺</t>
         </is>
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司推出1200万像素AI眼镜应用CMOS图像传感器SC1200IOT，官网还披露SC1200IOT/SC1220IOT具备小封装、低功耗、高感度、Always-On等特性，适用于AI眼镜及AR/VR微型摄像头模组；主板块保留AI眼镜CIS，跟踪量产客户和高像素新品。</t>
+          <t>证据中：2025年报披露维信诺围绕AI新场景推进智能终端、智能影像、智慧家居等显示供货，并持续推进ViP、Micro-LED等显示技术；真实受益节点是AI终端显示，MicroLED更多体现技术储备和参股生态。</t>
         </is>
       </c>
       <c r="E335" s="6" t="inlineStr">
@@ -9937,17 +9937,17 @@
       </c>
       <c r="B336" s="3" t="inlineStr">
         <is>
-          <t>688728</t>
+          <t>688213</t>
         </is>
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>格科微</t>
+          <t>思特威</t>
         </is>
       </c>
       <c r="D336" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司主营CIS与DDIC，高像素CIS放量；公告口径显示公司持续关注AI眼镜等新兴市场，500万和800万像素CIS已在AI眼镜项目量产。主板块保留AI眼镜CIS，但整体利润承压，需跟踪AI眼镜CIS是否能改善产品结构和毛利。</t>
+          <t>证据强：2025年报披露公司推出1200万像素AI眼镜应用CMOS图像传感器SC1200IOT，官网还披露SC1200IOT/SC1220IOT具备小封装、低功耗、高感度、Always-On等特性，适用于AI眼镜及AR/VR微型摄像头模组；主板块保留AI眼镜CIS，跟踪量产客户和高像素新品。</t>
         </is>
       </c>
       <c r="E336" s="6" t="inlineStr">
@@ -9959,22 +9959,22 @@
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜视觉算法</t>
+          <t>AI眼镜CIS</t>
         </is>
       </c>
       <c r="B337" s="3" t="inlineStr">
         <is>
-          <t>688088</t>
+          <t>688728</t>
         </is>
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>虹软科技</t>
+          <t>格科微</t>
         </is>
       </c>
       <c r="D337" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报/业绩快报披露AI眼镜影像与视觉算法持续升级，围绕复杂光照、动态场景、低照度和视频防抖推进平台适配；公开资料显示方案已在雷鸟、Rokid、夸克等AI眼镜落地。删减“端侧视觉AI底座”重复行，保留最直接的AI眼镜视觉算法。</t>
+          <t>证据中强：2025年报披露公司主营CIS与DDIC，高像素CIS放量；公告口径显示公司持续关注AI眼镜等新兴市场，500万和800万像素CIS已在AI眼镜项目量产。主板块保留AI眼镜CIS，但整体利润承压，需跟踪AI眼镜CIS是否能改善产品结构和毛利。</t>
         </is>
       </c>
       <c r="E337" s="6" t="inlineStr">
@@ -9986,22 +9986,22 @@
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜模拟芯片</t>
+          <t>AI眼镜视觉算法</t>
         </is>
       </c>
       <c r="B338" s="3" t="inlineStr">
         <is>
-          <t>688798</t>
+          <t>688088</t>
         </is>
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
-          <t>艾为电子</t>
+          <t>虹软科技</t>
         </is>
       </c>
       <c r="D338" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司高性能数模混合芯片覆盖音频功放、触觉反馈、马达驱动、压力/电容感应、灯效驱动等，SensorHub项目明确列示AI眼镜等IoT设备；另有AI眼镜客户导入音频功放、灯效驱动等公开信息。主板块保留AI眼镜模拟芯片，跟踪品牌客户放量和产品单机价值量。</t>
+          <t>证据强：2025年报/业绩快报披露AI眼镜影像与视觉算法持续升级，围绕复杂光照、动态场景、低照度和视频防抖推进平台适配；公开资料显示方案已在雷鸟、Rokid、夸克等AI眼镜落地。删减“端侧视觉AI底座”重复行，保留最直接的AI眼镜视觉算法。</t>
         </is>
       </c>
       <c r="E338" s="6" t="inlineStr">
@@ -10013,22 +10013,22 @@
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜声学传感器</t>
+          <t>AI眼镜模拟芯片</t>
         </is>
       </c>
       <c r="B339" s="3" t="inlineStr">
         <is>
-          <t>688286</t>
+          <t>688798</t>
         </is>
       </c>
       <c r="C339" s="2" t="inlineStr">
         <is>
-          <t>敏芯股份</t>
+          <t>艾为电子</t>
         </is>
       </c>
       <c r="D339" s="2" t="inlineStr">
         <is>
-          <t>证据中：公司提质增效报告披露布局高信噪比、低功耗数字麦克风，部分型号已小批量出货，并布局应用于AI眼镜的骨传导声学传感器；删减“高信噪比数字麦克风”重复行，合并为AI眼镜声学传感器。风险是AI眼镜相关产品仍处研发/小批量阶段，收入贡献未充分披露。</t>
+          <t>证据中强：2025年报披露公司高性能数模混合芯片覆盖音频功放、触觉反馈、马达驱动、压力/电容感应、灯效驱动等，SensorHub项目明确列示AI眼镜等IoT设备；另有AI眼镜客户导入音频功放、灯效驱动等公开信息。主板块保留AI眼镜模拟芯片，跟踪品牌客户放量和产品单机价值量。</t>
         </is>
       </c>
       <c r="E339" s="6" t="inlineStr">
@@ -10040,22 +10040,22 @@
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>消费锂电池</t>
+          <t>AI眼镜声学传感器</t>
         </is>
       </c>
       <c r="B340" s="3" t="inlineStr">
         <is>
-          <t>688772</t>
+          <t>688286</t>
         </is>
       </c>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>珠海冠宇</t>
+          <t>敏芯股份</t>
         </is>
       </c>
       <c r="D340" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司主营消费类锂离子电池，AI功能消费电子推出有望带来换机潮，消费类半固态电池已规模化量产；募集说明书提及智能手表、智能眼镜等可穿戴需求扩张。主板块保留消费锂电池，AI受益偏终端电池供能配套，直接度低于AI眼镜专用电池公司。</t>
+          <t>证据中：公司提质增效报告披露布局高信噪比、低功耗数字麦克风，部分型号已小批量出货，并布局应用于AI眼镜的骨传导声学传感器；删减“高信噪比数字麦克风”重复行，合并为AI眼镜声学传感器。风险是AI眼镜相关产品仍处研发/小批量阶段，收入贡献未充分披露。</t>
         </is>
       </c>
       <c r="E340" s="6" t="inlineStr">
@@ -10067,22 +10067,22 @@
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>AI智能眼镜电池</t>
+          <t>消费锂电池</t>
         </is>
       </c>
       <c r="B341" s="3" t="inlineStr">
         <is>
-          <t>001283</t>
+          <t>688772</t>
         </is>
       </c>
       <c r="C341" s="2" t="inlineStr">
         <is>
-          <t>豪鹏科技</t>
+          <t>珠海冠宇</t>
         </is>
       </c>
       <c r="D341" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报/公开资料披露公司布局AI智能眼镜电池，固态电池样品在AI终端、可穿戴设备等场景完成初步验证；删减“AI终端固态电池”重复行，当前主线仍是AI智能眼镜电池，固态电池属于下一代技术储备而非已验证主收入板块。</t>
+          <t>证据中：2025年报披露公司主营消费类锂离子电池，AI功能消费电子推出有望带来换机潮，消费类半固态电池已规模化量产；募集说明书提及智能手表、智能眼镜等可穿戴需求扩张。主板块保留消费锂电池，AI受益偏终端电池供能配套，直接度低于AI眼镜专用电池公司。</t>
         </is>
       </c>
       <c r="E341" s="6" t="inlineStr">
@@ -10094,22 +10094,22 @@
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>AI眼镜结构件</t>
+          <t>AI智能眼镜电池</t>
         </is>
       </c>
       <c r="B342" s="3" t="inlineStr">
         <is>
-          <t>300115</t>
+          <t>001283</t>
         </is>
       </c>
       <c r="C342" s="2" t="inlineStr">
         <is>
-          <t>长盈精密</t>
+          <t>豪鹏科技</t>
         </is>
       </c>
       <c r="D342" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报摘要披露公司抓住AI硬件迭代机遇，持续开发AI笔记本和可穿戴产品关键零部件，轻量化金属及非金属结构件取得突破；AI眼镜结构件面向头部客户是主要弹性来源。主板块保留AI眼镜结构件，风险是消费电子结构件仍具客户集中和价格压力。</t>
+          <t>证据中强：2025年报/公开资料披露公司布局AI智能眼镜电池，固态电池样品在AI终端、可穿戴设备等场景完成初步验证；删减“AI终端固态电池”重复行，当前主线仍是AI智能眼镜电池，固态电池属于下一代技术储备而非已验证主收入板块。</t>
         </is>
       </c>
       <c r="E342" s="6" t="inlineStr">
@@ -10121,22 +10121,22 @@
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>AI智能眼镜整机</t>
+          <t>AI眼镜结构件</t>
         </is>
       </c>
       <c r="B343" s="3" t="inlineStr">
         <is>
-          <t>002241</t>
+          <t>300115</t>
         </is>
       </c>
       <c r="C343" s="2" t="inlineStr">
         <is>
-          <t>歌尔股份</t>
+          <t>长盈精密</t>
         </is>
       </c>
       <c r="D343" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司研发围绕MEMS声学传感器、微系统模组、AI智能眼镜/AR光学器件、MR头显等，AI智能眼镜等新兴业务表现亮眼；作为精密零组件+整机制造平台，主板块保留AI智能眼镜整机，光学、声学、SiP模组作为支撑能力写入备注即可。风险是营收仍受传统消费电子/XR周期影响。</t>
+          <t>证据中强：2025年报摘要披露公司抓住AI硬件迭代机遇，持续开发AI笔记本和可穿戴产品关键零部件，轻量化金属及非金属结构件取得突破；AI眼镜结构件面向头部客户是主要弹性来源。主板块保留AI眼镜结构件，风险是消费电子结构件仍具客户集中和价格压力。</t>
         </is>
       </c>
       <c r="E343" s="6" t="inlineStr">
@@ -10148,22 +10148,22 @@
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>AI终端精密功能件</t>
+          <t>AI智能眼镜整机</t>
         </is>
       </c>
       <c r="B344" s="3" t="inlineStr">
         <is>
-          <t>002600</t>
+          <t>002241</t>
         </is>
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>领益智造</t>
+          <t>歌尔股份</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报摘要披露公司核心产品覆盖AI手机、AIPC、AI眼镜及XR可穿戴、AI服务器、机器人等硬件，以2024年收入计在全球AI终端高精密功能件行业排名第一；半年报披露AR眼镜项目含MicroOLED显示、Insert Molding金属件增强等。主板块从精密结构件扩展为AI终端精密功能件。</t>
+          <t>证据中强：2025年报披露公司研发围绕MEMS声学传感器、微系统模组、AI智能眼镜/AR光学器件、MR头显等，AI智能眼镜等新兴业务表现亮眼；作为精密零组件+整机制造平台，主板块保留AI智能眼镜整机，光学、声学、SiP模组作为支撑能力写入备注即可。风险是营收仍受传统消费电子/XR周期影响。</t>
         </is>
       </c>
       <c r="E344" s="6" t="inlineStr">
@@ -10175,22 +10175,22 @@
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>机器人3D视觉</t>
+          <t>AI终端精密功能件</t>
         </is>
       </c>
       <c r="B345" s="3" t="inlineStr">
         <is>
-          <t>688322</t>
+          <t>002600</t>
         </is>
       </c>
       <c r="C345" s="2" t="inlineStr">
         <is>
-          <t>奥比中光</t>
+          <t>领益智造</t>
         </is>
       </c>
       <c r="D345" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司专注3D视觉感知，在人工智能与机器人时代打造“机器人之眼”和机器人与AI视觉产业中台；产品和生态围绕机器人、AI视觉、3D相机矩阵推进。删减泛化的“3D视觉传感器”重复表述，主板块保留机器人3D视觉。风险是机器人需求仍处导入期，短期收入仍含AIoT/生物识别等多场景。</t>
+          <t>证据强：2025年报摘要披露公司核心产品覆盖AI手机、AIPC、AI眼镜及XR可穿戴、AI服务器、机器人等硬件，以2024年收入计在全球AI终端高精密功能件行业排名第一；半年报披露AR眼镜项目含MicroOLED显示、Insert Molding金属件增强等。主板块从精密结构件扩展为AI终端精密功能件。</t>
         </is>
       </c>
       <c r="E345" s="6" t="inlineStr">
@@ -10202,22 +10202,22 @@
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>机器人力传感器</t>
+          <t>机器人3D视觉</t>
         </is>
       </c>
       <c r="B346" s="3" t="inlineStr">
         <is>
-          <t>603662</t>
+          <t>688322</t>
         </is>
       </c>
       <c r="C346" s="2" t="inlineStr">
         <is>
-          <t>柯力传感</t>
+          <t>奥比中光</t>
         </is>
       </c>
       <c r="D346" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司围绕人形、协作和工业机器人加快六维力/力矩、一维至三维力、触觉、IMU等产品研发认证及批量交付；半年报披露以六维力/力矩为核心融合触觉、IMU的机器人传感方案。删减“触觉传感器-IMU”重复行，保留最能解释AI机器人弹性的机器人力传感器。</t>
+          <t>证据强：2025年报披露公司专注3D视觉感知，在人工智能与机器人时代打造“机器人之眼”和机器人与AI视觉产业中台；产品和生态围绕机器人、AI视觉、3D相机矩阵推进。删减泛化的“3D视觉传感器”重复表述，主板块保留机器人3D视觉。风险是机器人需求仍处导入期，短期收入仍含AIoT/生物识别等多场景。</t>
         </is>
       </c>
       <c r="E346" s="6" t="inlineStr">
@@ -10234,17 +10234,17 @@
       </c>
       <c r="B347" s="3" t="inlineStr">
         <is>
-          <t>301413</t>
+          <t>603662</t>
         </is>
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>安培龙</t>
+          <t>柯力传感</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报/投资者关系披露公司机器人力传感器包括单向力、力矩及六维力传感器，基于MEMS硅基应变片和玻璃微熔工艺的单向力及力矩传感器已开发完成并向多家机器人客户送样。主板块保留机器人力传感器，但公告提示相关收入占比仍低，六维力部分仍需验证批量订单。</t>
+          <t>证据强：2025年报披露公司围绕人形、协作和工业机器人加快六维力/力矩、一维至三维力、触觉、IMU等产品研发认证及批量交付；半年报披露以六维力/力矩为核心融合触觉、IMU的机器人传感方案。删减“触觉传感器-IMU”重复行，保留最能解释AI机器人弹性的机器人力传感器。</t>
         </is>
       </c>
       <c r="E347" s="6" t="inlineStr">
@@ -10261,17 +10261,17 @@
       </c>
       <c r="B348" s="3" t="inlineStr">
         <is>
-          <t>300354</t>
+          <t>301413</t>
         </is>
       </c>
       <c r="C348" s="2" t="inlineStr">
         <is>
-          <t>东华测试</t>
+          <t>安培龙</t>
         </is>
       </c>
       <c r="D348" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025投资者关系记录披露六维力传感器处于小批量试制阶段，下游包括工业机器人、人形机器人、航空航天、汽车、电子、医疗等；公司主业仍以结构力学性能测试、PHM、电化学工作站等为基础，机器人收入贡献尚未充分披露，跟踪送样转批量和标定/测试体系能力。</t>
+          <t>证据中：2025年报/投资者关系披露公司机器人力传感器包括单向力、力矩及六维力传感器，基于MEMS硅基应变片和玻璃微熔工艺的单向力及力矩传感器已开发完成并向多家机器人客户送样。主板块保留机器人力传感器，但公告提示相关收入占比仍低，六维力部分仍需验证批量订单。</t>
         </is>
       </c>
       <c r="E348" s="6" t="inlineStr">
@@ -10283,22 +10283,22 @@
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>机器人电子皮肤</t>
+          <t>机器人力传感器</t>
         </is>
       </c>
       <c r="B349" s="3" t="inlineStr">
         <is>
-          <t>300007</t>
+          <t>300354</t>
         </is>
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>汉威科技</t>
+          <t>东华测试</t>
         </is>
       </c>
       <c r="D349" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露柔性传感电子皮肤入选2025具身智能十大创新产品和技术，机器人相关电子皮肤和触觉传感器已小批量供货；公司官网披露具备年产1000万支柔性传感器产线和柔性压阻/压电/电容/汗液四大技术。主板块从电子皮肤规范为机器人电子皮肤，风险是整体业务仍以气体/仪表等传感平台为主。</t>
+          <t>证据中：2025投资者关系记录披露六维力传感器处于小批量试制阶段，下游包括工业机器人、人形机器人、航空航天、汽车、电子、医疗等；公司主业仍以结构力学性能测试、PHM、电化学工作站等为基础，机器人收入贡献尚未充分披露，跟踪送样转批量和标定/测试体系能力。</t>
         </is>
       </c>
       <c r="E349" s="6" t="inlineStr">
@@ -10310,22 +10310,22 @@
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>机器人谐波减速器</t>
+          <t>机器人电子皮肤</t>
         </is>
       </c>
       <c r="B350" s="3" t="inlineStr">
         <is>
-          <t>688017</t>
+          <t>300007</t>
         </is>
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>绿的谐波</t>
+          <t>汉威科技</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司巩固具身智能场景谐波减速器领先地位，并围绕轻量化、微型化、低噪音、精度、刚性和寿命持续攻关；同时突破行星滚柱丝杠规模化制造并扩展直线伺服关节。主板块从泛机器人执行器收敛为机器人谐波减速器，丝杠和机电一体化作为增量能力跟踪。</t>
+          <t>证据强：2025年报披露柔性传感电子皮肤入选2025具身智能十大创新产品和技术，机器人相关电子皮肤和触觉传感器已小批量供货；公司官网披露具备年产1000万支柔性传感器产线和柔性压阻/压电/电容/汗液四大技术。主板块从电子皮肤规范为机器人电子皮肤，风险是整体业务仍以气体/仪表等传感平台为主。</t>
         </is>
       </c>
       <c r="E350" s="6" t="inlineStr">
@@ -10337,22 +10337,22 @@
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>机器人精密减速器</t>
+          <t>机器人谐波减速器</t>
         </is>
       </c>
       <c r="B351" s="3" t="inlineStr">
         <is>
-          <t>002896</t>
+          <t>688017</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>中大力德</t>
+          <t>绿的谐波</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露精密减速器受工业机器人产量增长、人形机器人原型机批量落地等带动，公司具备行星、RV、谐波三大减速器布局，并通过减速器+电机+驱动一体化架构形成智能执行单元。主板块从机器人减速器规范为机器人精密减速器，跟踪人形机器人客户、型号验证和毛利率。</t>
+          <t>证据强：2025年报披露公司巩固具身智能场景谐波减速器领先地位，并围绕轻量化、微型化、低噪音、精度、刚性和寿命持续攻关；同时突破行星滚柱丝杠规模化制造并扩展直线伺服关节。主板块从泛机器人执行器收敛为机器人谐波减速器，丝杠和机电一体化作为增量能力跟踪。</t>
         </is>
       </c>
       <c r="E351" s="6" t="inlineStr">
@@ -10369,17 +10369,17 @@
       </c>
       <c r="B352" s="3" t="inlineStr">
         <is>
-          <t>002472</t>
+          <t>002896</t>
         </is>
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>双环传动</t>
+          <t>中大力德</t>
         </is>
       </c>
       <c r="D352" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露工业机器人核心零部件减速器趋势向好，公司在重载RV精密减速器领域攻克高精度、长寿命核心技术；控股子公司从事机器人关节高精密减速器研发生产，产品包括RV减速器、精密配件及谐波减速器。主板块从机器人减速器细化为机器人高精密减速器，风险是汽车齿轮仍是主要利润来源。</t>
+          <t>证据中强：2025年报披露精密减速器受工业机器人产量增长、人形机器人原型机批量落地等带动，公司具备行星、RV、谐波三大减速器布局，并通过减速器+电机+驱动一体化架构形成智能执行单元。主板块从机器人减速器规范为机器人精密减速器，跟踪人形机器人客户、型号验证和毛利率。</t>
         </is>
       </c>
       <c r="E352" s="6" t="inlineStr">
@@ -10391,22 +10391,22 @@
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>行星滚柱丝杠</t>
+          <t>机器人精密减速器</t>
         </is>
       </c>
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>603667</t>
+          <t>002472</t>
         </is>
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>五洲新春</t>
+          <t>双环传动</t>
         </is>
       </c>
       <c r="D353" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025定增预案披露具身智能机器人和汽车智驾核心零部件项目，达产后规划年产98万套行星滚柱丝杠、210万套微型滚珠丝杠和7万组通用机器人专用轴承；删减机器人专用轴承重复行，保留最能解释人形机器人弹性的行星滚柱丝杠。风险是募投建设周期较长，当前丝杠收入基数仍小。</t>
+          <t>证据中强：2025年报披露工业机器人核心零部件减速器趋势向好，公司在重载RV精密减速器领域攻克高精度、长寿命核心技术；控股子公司从事机器人关节高精密减速器研发生产，产品包括RV减速器、精密配件及谐波减速器。主板块从机器人减速器细化为机器人高精密减速器，风险是汽车齿轮仍是主要利润来源。</t>
         </is>
       </c>
       <c r="E353" s="6" t="inlineStr">
@@ -10423,17 +10423,17 @@
       </c>
       <c r="B354" s="3" t="inlineStr">
         <is>
-          <t>601100</t>
+          <t>603667</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>恒立液压</t>
+          <t>五洲新春</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露线性驱动项目投产，精密丝杠、直线导轨、电动缸等产品拓展；行星滚柱丝杠已完成送样和初步量产，为精密传动业务开拓机器人等多元下游市场。主板块保留行星滚柱丝杠，但公司基本盘仍是液压件，机器人弹性需看丝杠客户验证、量产节奏和收入占比。</t>
+          <t>证据中强：2025定增预案披露具身智能机器人和汽车智驾核心零部件项目，达产后规划年产98万套行星滚柱丝杠、210万套微型滚珠丝杠和7万组通用机器人专用轴承；删减机器人专用轴承重复行，保留最能解释人形机器人弹性的行星滚柱丝杠。风险是募投建设周期较长，当前丝杠收入基数仍小。</t>
         </is>
       </c>
       <c r="E354" s="6" t="inlineStr">
@@ -10450,17 +10450,17 @@
       </c>
       <c r="B355" s="3" t="inlineStr">
         <is>
-          <t>688678</t>
+          <t>601100</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>福立旺</t>
+          <t>恒立液压</t>
         </is>
       </c>
       <c r="D355" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025提质增效评估/公开资料披露公司向人形机器人精密传动拓展，已开发5.0mm、6.5mm、9.0mm等螺母直径规格微型行星滚柱丝杠，并向多家头部客户送样；删减机器人关节结构件重复行，关节护罩、驱动器支架等结构件作为补充交付能力。风险是主业仍为精密金属零部件，丝杠商业化仍早期。</t>
+          <t>证据中：2025年报披露线性驱动项目投产，精密丝杠、直线导轨、电动缸等产品拓展；行星滚柱丝杠已完成送样和初步量产，为精密传动业务开拓机器人等多元下游市场。主板块保留行星滚柱丝杠，但公司基本盘仍是液压件，机器人弹性需看丝杠客户验证、量产节奏和收入占比。</t>
         </is>
       </c>
       <c r="E355" s="6" t="inlineStr">
@@ -10477,17 +10477,17 @@
       </c>
       <c r="B356" s="3" t="inlineStr">
         <is>
-          <t>603009</t>
+          <t>688678</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>北特科技</t>
+          <t>福立旺</t>
         </is>
       </c>
       <c r="D356" s="2" t="inlineStr">
         <is>
-          <t>证据中强：募集说明书披露差动式行星滚柱丝杠承载能力强、刚度大、磨损小和寿命长，适用于高负载线性执行场合；募投项目达产后规划年产80万套行星滚柱丝杠，主要应用于人形机器人肢体线性运动。主板块保留差动式行星滚柱丝杠，风险是募投产能释放和客户量产验证仍需跟踪。</t>
+          <t>证据中：2025提质增效评估/公开资料披露公司向人形机器人精密传动拓展，已开发5.0mm、6.5mm、9.0mm等螺母直径规格微型行星滚柱丝杠，并向多家头部客户送样；删减机器人关节结构件重复行，关节护罩、驱动器支架等结构件作为补充交付能力。风险是主业仍为精密金属零部件，丝杠商业化仍早期。</t>
         </is>
       </c>
       <c r="E356" s="6" t="inlineStr">
@@ -10499,22 +10499,22 @@
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>机器人执行器</t>
+          <t>行星滚柱丝杠</t>
         </is>
       </c>
       <c r="B357" s="3" t="inlineStr">
         <is>
-          <t>601689</t>
+          <t>603009</t>
         </is>
       </c>
       <c r="C357" s="2" t="inlineStr">
         <is>
-          <t>拓普集团</t>
+          <t>北特科技</t>
         </is>
       </c>
       <c r="D357" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司已设立机器人执行器事业部，布局直线执行器、旋转执行器、灵巧手、传感器、躯体结构件、足部减震器、电子柔性皮肤等平台化产品；直线执行器获得客户认可后继续送样旋转执行器和灵巧手电机。主板块保留机器人执行器，风险是收入主体仍为汽车零部件且机器人客户/订单未完全披露。</t>
+          <t>证据中强：募集说明书披露差动式行星滚柱丝杠承载能力强、刚度大、磨损小和寿命长，适用于高负载线性执行场合；募投项目达产后规划年产80万套行星滚柱丝杠，主要应用于人形机器人肢体线性运动。主板块保留差动式行星滚柱丝杠，风险是募投产能释放和客户量产验证仍需跟踪。</t>
         </is>
       </c>
       <c r="E357" s="6" t="inlineStr">
@@ -10526,22 +10526,22 @@
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>机器人伺服驱动</t>
+          <t>机器人执行器</t>
         </is>
       </c>
       <c r="B358" s="3" t="inlineStr">
         <is>
-          <t>300124</t>
+          <t>601689</t>
         </is>
       </c>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>汇川技术</t>
+          <t>拓普集团</t>
         </is>
       </c>
       <c r="D358" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露人形机器人业务已完成从预研到商业化突破，构建核心部件全栈能力，完成无框力矩电机、低压高功率伺服驱动器、关节模组、行星滚柱丝杠、编码器等第一代产品开发和交付；删减“机器人直线导轨-丝杠”重复行，保留最能体现汇川运动控制优势的机器人伺服驱动。</t>
+          <t>证据中强：2025年报披露公司已设立机器人执行器事业部，布局直线执行器、旋转执行器、灵巧手、传感器、躯体结构件、足部减震器、电子柔性皮肤等平台化产品；直线执行器获得客户认可后继续送样旋转执行器和灵巧手电机。主板块保留机器人执行器，风险是收入主体仍为汽车零部件且机器人客户/订单未完全披露。</t>
         </is>
       </c>
       <c r="E358" s="6" t="inlineStr">
@@ -10553,22 +10553,22 @@
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>机器人驱控系统</t>
+          <t>机器人伺服驱动</t>
         </is>
       </c>
       <c r="B359" s="3" t="inlineStr">
         <is>
-          <t>002979</t>
+          <t>300124</t>
         </is>
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
-          <t>雷赛智能</t>
+          <t>汇川技术</t>
         </is>
       </c>
       <c r="D359" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司机器人核心部件覆盖高密度无框力矩电机、中空编码器、空心杯电机、微型伺服、谐波/行星关节模组、高中低自由度灵巧手，并布局运动控制“小脑”；关节模组与灵巧手已进入数十家主流客户批量供货。主板块从机器人关节运动控制收敛为机器人驱控系统。</t>
+          <t>证据强：2025年报披露人形机器人业务已完成从预研到商业化突破，构建核心部件全栈能力，完成无框力矩电机、低压高功率伺服驱动器、关节模组、行星滚柱丝杠、编码器等第一代产品开发和交付；删减“机器人直线导轨-丝杠”重复行，保留最能体现汇川运动控制优势的机器人伺服驱动。</t>
         </is>
       </c>
       <c r="E359" s="6" t="inlineStr">
@@ -10580,22 +10580,22 @@
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>空心杯电机</t>
+          <t>机器人驱控系统</t>
         </is>
       </c>
       <c r="B360" s="3" t="inlineStr">
         <is>
-          <t>603728</t>
+          <t>002979</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>鸣志电器</t>
+          <t>雷赛智能</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露无刷电机模组、无齿槽空心杯模组、无框/交流伺服电机及驱动控制系统、精密减速机和丝杠传动模组广泛适用于人形机器人灵巧手、关节、底盘等；删减“运动控制”重复行，保留最具人形机器人弹性的空心杯电机，运动控制平台作为配套能力。</t>
+          <t>证据强：2025年报披露公司机器人核心部件覆盖高密度无框力矩电机、中空编码器、空心杯电机、微型伺服、谐波/行星关节模组、高中低自由度灵巧手，并布局运动控制“小脑”；关节模组与灵巧手已进入数十家主流客户批量供货。主板块从机器人关节运动控制收敛为机器人驱控系统。</t>
         </is>
       </c>
       <c r="E360" s="6" t="inlineStr">
@@ -10607,22 +10607,22 @@
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>行业大模型+Agent平台</t>
+          <t>空心杯电机</t>
         </is>
       </c>
       <c r="B361" s="3" t="inlineStr">
         <is>
-          <t>300229</t>
+          <t>603728</t>
         </is>
       </c>
       <c r="C361" s="2" t="inlineStr">
         <is>
-          <t>拓尔思</t>
+          <t>鸣志电器</t>
         </is>
       </c>
       <c r="D361" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025半年报/公告披露高质量数据集系统、海贝搜索向量数据库、拓天链Agent平台及拓天大模型等；数据和向量数据库是底座，商业化主线为行业大模型+Agent平台。</t>
+          <t>证据强：2025年报披露无刷电机模组、无齿槽空心杯模组、无框/交流伺服电机及驱动控制系统、精密减速机和丝杠传动模组广泛适用于人形机器人灵巧手、关节、底盘等；删减“运动控制”重复行，保留最具人形机器人弹性的空心杯电机，运动控制平台作为配套能力。</t>
         </is>
       </c>
       <c r="E361" s="6" t="inlineStr">
@@ -10634,22 +10634,22 @@
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>行业大模型训推一体</t>
+          <t>行业大模型+Agent平台</t>
         </is>
       </c>
       <c r="B362" s="3" t="inlineStr">
         <is>
-          <t>688327</t>
+          <t>300229</t>
         </is>
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>云从科技</t>
+          <t>拓尔思</t>
         </is>
       </c>
       <c r="D362" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司基于CWOS和从容多模态大模型推出大模型训推及智用一体机，并在工程、制造、政务等场景落地；多模态大模型是底座，主线收敛为行业大模型训推一体。</t>
+          <t>证据强：2025半年报/公告披露高质量数据集系统、海贝搜索向量数据库、拓天链Agent平台及拓天大模型等；数据和向量数据库是底座，商业化主线为行业大模型+Agent平台。</t>
         </is>
       </c>
       <c r="E362" s="6" t="inlineStr">
@@ -10661,22 +10661,22 @@
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>国产算力大模型底座</t>
+          <t>行业大模型训推一体</t>
         </is>
       </c>
       <c r="B363" s="3" t="inlineStr">
         <is>
-          <t>002230</t>
+          <t>688327</t>
         </is>
       </c>
       <c r="C363" s="2" t="inlineStr">
         <is>
-          <t>科大讯飞</t>
+          <t>云从科技</t>
         </is>
       </c>
       <c r="D363" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露讯飞星火持续基于全国产算力训练并推进X1/X1.5等推理模型，2025年大模型相关项目中标金额领先；行业大模型与AI开放平台是商业化路径，合并降级到备注。</t>
+          <t>证据中强：2025年报披露公司基于CWOS和从容多模态大模型推出大模型训推及智用一体机，并在工程、制造、政务等场景落地；多模态大模型是底座，主线收敛为行业大模型训推一体。</t>
         </is>
       </c>
       <c r="E363" s="6" t="inlineStr">
@@ -10688,22 +10688,22 @@
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>企业AI平台</t>
+          <t>国产算力大模型底座</t>
         </is>
       </c>
       <c r="B364" s="3" t="inlineStr">
         <is>
-          <t>600588</t>
+          <t>002230</t>
         </is>
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>用友网络</t>
+          <t>科大讯飞</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露用友BIP以AI×数据×流程原生一体，将企业AI融入财务、人力、供应链、制造等核心业务；但公司仍亏损，主线保留企业AI平台并提示盈利修复风险。</t>
+          <t>证据强：2025年报披露讯飞星火持续基于全国产算力训练并推进X1/X1.5等推理模型，2025年大模型相关项目中标金额领先；行业大模型与AI开放平台是商业化路径，合并降级到备注。</t>
         </is>
       </c>
       <c r="E364" s="6" t="inlineStr">
@@ -10715,22 +10715,22 @@
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>企业级AI应用平台</t>
+          <t>企业AI平台</t>
         </is>
       </c>
       <c r="B365" s="3" t="inlineStr">
         <is>
-          <t>300170</t>
+          <t>600588</t>
         </is>
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>汉得信息</t>
+          <t>用友网络</t>
         </is>
       </c>
       <c r="D365" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司加大行业大模型和垂类智能体研发，基于H-ZERO、H-ONE构建企业级AI基础设施并打造AI应用工厂；AI业务收入放量，主板块由企业AI中台升级为企业级AI应用平台。</t>
+          <t>证据中强：2025年报披露用友BIP以AI×数据×流程原生一体，将企业AI融入财务、人力、供应链、制造等核心业务；但公司仍亏损，主线保留企业AI平台并提示盈利修复风险。</t>
         </is>
       </c>
       <c r="E365" s="6" t="inlineStr">
@@ -10742,22 +10742,22 @@
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>行业AI智能体平台</t>
+          <t>企业级AI应用平台</t>
         </is>
       </c>
       <c r="B366" s="3" t="inlineStr">
         <is>
-          <t>301236</t>
+          <t>300170</t>
         </is>
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>软通动力</t>
+          <t>汉得信息</t>
         </is>
       </c>
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司以软通天璇AutoAgent等平台为引擎，提供从AI咨询、模型部署、智能体开发到持续运营的全流程智能化升级服务；主板块保留行业AI平台并细化为行业AI智能体平台。</t>
+          <t>证据强：2025年报披露公司加大行业大模型和垂类智能体研发，基于H-ZERO、H-ONE构建企业级AI基础设施并打造AI应用工厂；AI业务收入放量，主板块由企业AI中台升级为企业级AI应用平台。</t>
         </is>
       </c>
       <c r="E366" s="6" t="inlineStr">
@@ -10769,22 +10769,22 @@
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>制造业AI智能体平台</t>
+          <t>行业AI智能体平台</t>
         </is>
       </c>
       <c r="B367" s="3" t="inlineStr">
         <is>
-          <t>300378</t>
+          <t>301236</t>
         </is>
       </c>
       <c r="C367" s="2" t="inlineStr">
         <is>
-          <t>鼎捷数智</t>
+          <t>软通动力</t>
         </is>
       </c>
       <c r="D367" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司持续升级鼎捷雅典娜数智底座并丰富AI智能体矩阵，AI相关业务签约金额近2亿元，覆盖生产、销售、财务等制造场景；主板块由工业AI细化为制造业AI智能体平台。</t>
+          <t>证据强：2025年报披露公司以软通天璇AutoAgent等平台为引擎，提供从AI咨询、模型部署、智能体开发到持续运营的全流程智能化升级服务；主板块保留行业AI平台并细化为行业AI智能体平台。</t>
         </is>
       </c>
       <c r="E367" s="6" t="inlineStr">
@@ -10796,22 +10796,22 @@
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>行业AI交付</t>
+          <t>制造业AI智能体平台</t>
         </is>
       </c>
       <c r="B368" s="3" t="inlineStr">
         <is>
-          <t>002649</t>
+          <t>300378</t>
         </is>
       </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>博彦科技</t>
+          <t>鼎捷数智</t>
         </is>
       </c>
       <c r="D368" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以AI、大数据为技术底座，依托人工智能计算平台和AI Agent平台，在金融、能源、化工等行业提供AI咨询、解决方案、实施与运营；AI中台是能力底座，合并到行业AI交付。</t>
+          <t>证据强：2025年报披露公司持续升级鼎捷雅典娜数智底座并丰富AI智能体矩阵，AI相关业务签约金额近2亿元，覆盖生产、销售、财务等制造场景；主板块由工业AI细化为制造业AI智能体平台。</t>
         </is>
       </c>
       <c r="E368" s="6" t="inlineStr">
@@ -10823,22 +10823,22 @@
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>AI数据基础设施软件</t>
+          <t>行业AI交付</t>
         </is>
       </c>
       <c r="B369" s="3" t="inlineStr">
         <is>
-          <t>688031</t>
+          <t>002649</t>
         </is>
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
-          <t>星环科技</t>
+          <t>博彦科技</t>
         </is>
       </c>
       <c r="D369" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报显示公司定位企业级AI和大数据基础设施软件，覆盖大数据平台、分布式数据库、数据开发工具和AI平台，并参与向量数据库标准；AI加速卡池化更像数据库/GPU加速能力，合并降级到备注。</t>
+          <t>证据中强：2025年报披露公司以AI、大数据为技术底座，依托人工智能计算平台和AI Agent平台，在金融、能源、化工等行业提供AI咨询、解决方案、实施与运营；AI中台是能力底座，合并到行业AI交付。</t>
         </is>
       </c>
       <c r="E369" s="6" t="inlineStr">
@@ -10850,22 +10850,22 @@
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>向量数据库</t>
+          <t>AI数据基础设施软件</t>
         </is>
       </c>
       <c r="B370" s="3" t="inlineStr">
         <is>
-          <t>603138</t>
+          <t>688031</t>
         </is>
       </c>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>海量数据</t>
+          <t>星环科技</t>
         </is>
       </c>
       <c r="D370" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司专注数据库，Vastbase与向量数据库等AI相关能力是大模型开发和智能问答等场景底座；但收入仍以国产数据库替代为主，向量数据库商业化占比未充分拆分。</t>
+          <t>证据中强：2025年报显示公司定位企业级AI和大数据基础设施软件，覆盖大数据平台、分布式数据库、数据开发工具和AI平台，并参与向量数据库标准；AI加速卡池化更像数据库/GPU加速能力，合并降级到备注。</t>
         </is>
       </c>
       <c r="E370" s="6" t="inlineStr">
@@ -10877,22 +10877,22 @@
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>AI数据库</t>
+          <t>向量数据库</t>
         </is>
       </c>
       <c r="B371" s="3" t="inlineStr">
         <is>
-          <t>688692</t>
+          <t>603138</t>
         </is>
       </c>
       <c r="C371" s="2" t="inlineStr">
         <is>
-          <t>达梦数据</t>
+          <t>海量数据</t>
         </is>
       </c>
       <c r="D371" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报显示软件产品使用授权仍是核心收入引擎，公司围绕数据库、云计算、大数据、AI相关产品和数据库一体机形成全栈布局；合并“全栈数据产品”，主板块保留AI数据库。</t>
+          <t>证据中：2025年报披露公司专注数据库，Vastbase与向量数据库等AI相关能力是大模型开发和智能问答等场景底座；但收入仍以国产数据库替代为主，向量数据库商业化占比未充分拆分。</t>
         </is>
       </c>
       <c r="E371" s="6" t="inlineStr">
@@ -10904,22 +10904,22 @@
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>多模态训练数据</t>
+          <t>AI数据库</t>
         </is>
       </c>
       <c r="B372" s="3" t="inlineStr">
         <is>
-          <t>688787</t>
+          <t>688692</t>
         </is>
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>海天瑞声</t>
+          <t>达梦数据</t>
         </is>
       </c>
       <c r="D372" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露全球AI渗透和多模态大模型需求推动训练数据服务扩容，公司持续投入语音、视觉、NLP、3D点云及大模型数据清洗/自动标注能力；主板块由训练数据细化为多模态训练数据。</t>
+          <t>证据强：2025年报显示软件产品使用授权仍是核心收入引擎，公司围绕数据库、云计算、大数据、AI相关产品和数据库一体机形成全栈布局；合并“全栈数据产品”，主板块保留AI数据库。</t>
         </is>
       </c>
       <c r="E372" s="6" t="inlineStr">
@@ -10931,22 +10931,22 @@
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>中文数据语料</t>
+          <t>多模态训练数据</t>
         </is>
       </c>
       <c r="B373" s="3" t="inlineStr">
         <is>
-          <t>688228</t>
+          <t>688787</t>
         </is>
       </c>
       <c r="C373" s="2" t="inlineStr">
         <is>
-          <t>开普云</t>
+          <t>海天瑞声</t>
         </is>
       </c>
       <c r="D373" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司积累PB级数据并参与中文互联网基础语料3.0，专题数据语料平台仍处产品开发阶段；AI链逻辑存在，但商业化确定性低于成熟软件/SaaS。</t>
+          <t>证据强：2025年报披露全球AI渗透和多模态大模型需求推动训练数据服务扩容，公司持续投入语音、视觉、NLP、3D点云及大模型数据清洗/自动标注能力；主板块由训练数据细化为多模态训练数据。</t>
         </is>
       </c>
       <c r="E373" s="6" t="inlineStr">
@@ -10958,22 +10958,22 @@
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>AI安全</t>
+          <t>中文数据语料</t>
         </is>
       </c>
       <c r="B374" s="3" t="inlineStr">
         <is>
-          <t>002439</t>
+          <t>688228</t>
         </is>
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>启明星辰</t>
+          <t>开普云</t>
         </is>
       </c>
       <c r="D374" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露以AI+安全为核心，推出大模型应用防火墙、访问安全代理、评估系统、脱敏罩、水印及拦截清洗等矩阵；由泛AI安全收敛为大模型应用安全防护。</t>
+          <t>证据中：2025年报披露公司积累PB级数据并参与中文互联网基础语料3.0，专题数据语料平台仍处产品开发阶段；AI链逻辑存在，但商业化确定性低于成熟软件/SaaS。</t>
         </is>
       </c>
       <c r="E374" s="6" t="inlineStr">
@@ -10990,17 +10990,17 @@
       </c>
       <c r="B375" s="3" t="inlineStr">
         <is>
-          <t>300454</t>
+          <t>002439</t>
         </is>
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>深信服</t>
+          <t>启明星辰</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露AI安全平台以安全数据和模型底座为核心，结合安全GPT大模型，覆盖安全运营、零信任、数据安全、终端安全；AI算力网关和办公助手为辅线。</t>
+          <t>证据强：2025年报披露以AI+安全为核心，推出大模型应用防火墙、访问安全代理、评估系统、脱敏罩、水印及拦截清洗等矩阵；由泛AI安全收敛为大模型应用安全防护。</t>
         </is>
       </c>
       <c r="E375" s="6" t="inlineStr">
@@ -11017,17 +11017,17 @@
       </c>
       <c r="B376" s="3" t="inlineStr">
         <is>
-          <t>688561</t>
+          <t>300454</t>
         </is>
       </c>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t>奇安信</t>
+          <t>深信服</t>
         </is>
       </c>
       <c r="D376" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露AISOC、AI+代码卫士、大模型卫士等AI安全新品在客户侧验证并转化收入，覆盖安全运营、检测、数据、代码、攻防智能体；由泛AI安全收敛为AI安全智能体。</t>
+          <t>证据强：2025年报披露AI安全平台以安全数据和模型底座为核心，结合安全GPT大模型，覆盖安全运营、零信任、数据安全、终端安全；AI算力网关和办公助手为辅线。</t>
         </is>
       </c>
       <c r="E376" s="6" t="inlineStr">
@@ -11044,17 +11044,17 @@
       </c>
       <c r="B377" s="3" t="inlineStr">
         <is>
-          <t>688023</t>
+          <t>688561</t>
         </is>
       </c>
       <c r="C377" s="2" t="inlineStr">
         <is>
-          <t>安恒信息</t>
+          <t>奇安信</t>
         </is>
       </c>
       <c r="D377" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露恒脑安全垂域大模型支持多参数模型、量化、软硬一体/SaaS交付并上线智能体商城；AI数据分类分级是恒脑体系的应用场景，合并降级到备注。</t>
+          <t>证据强：2025年报披露AISOC、AI+代码卫士、大模型卫士等AI安全新品在客户侧验证并转化收入，覆盖安全运营、检测、数据、代码、攻防智能体；由泛AI安全收敛为AI安全智能体。</t>
         </is>
       </c>
       <c r="E377" s="6" t="inlineStr">
@@ -11071,17 +11071,17 @@
       </c>
       <c r="B378" s="3" t="inlineStr">
         <is>
-          <t>601360</t>
+          <t>688023</t>
         </is>
       </c>
       <c r="C378" s="2" t="inlineStr">
         <is>
-          <t>三六零</t>
+          <t>安恒信息</t>
         </is>
       </c>
       <c r="D378" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报/半年报披露自研AI大模型驱动互联网产品，同时360安全大模型已在大量用户真实环境测试、应用与交付；主板块由宽泛360大模型收敛为360安全大模型。</t>
+          <t>证据强：2025年报披露恒脑安全垂域大模型支持多参数模型、量化、软硬一体/SaaS交付并上线智能体商城；AI数据分类分级是恒脑体系的应用场景，合并降级到备注。</t>
         </is>
       </c>
       <c r="E378" s="6" t="inlineStr">
@@ -11098,17 +11098,17 @@
       </c>
       <c r="B379" s="3" t="inlineStr">
         <is>
-          <t>300369</t>
+          <t>601360</t>
         </is>
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
-          <t>绿盟科技</t>
+          <t>三六零</t>
         </is>
       </c>
       <c r="D379" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露清风卫AI安全系列覆盖评估、防护、响应，并推出AI全生命周期安全测评和备案服务，国家级攻防演练AI内容安全赛道表现突出；保留清风卫AI安全。</t>
+          <t>证据中强：2025年报/半年报披露自研AI大模型驱动互联网产品，同时360安全大模型已在大量用户真实环境测试、应用与交付；主板块由宽泛360大模型收敛为360安全大模型。</t>
         </is>
       </c>
       <c r="E379" s="6" t="inlineStr">
@@ -11120,22 +11120,22 @@
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>AI办公Agent</t>
+          <t>AI安全</t>
         </is>
       </c>
       <c r="B380" s="3" t="inlineStr">
         <is>
-          <t>688111</t>
+          <t>300369</t>
         </is>
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>金山办公</t>
+          <t>绿盟科技</t>
         </is>
       </c>
       <c r="D380" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露WPS AI政务版、企业知识库、可信溯源和私有化部署等能力，WPS 365持续向企业级智能办公平台演进；企业知识库是AI办公Agent底座能力，合并到备注。</t>
+          <t>证据强：2025年报披露清风卫AI安全系列覆盖评估、防护、响应，并推出AI全生命周期安全测评和备案服务，国家级攻防演练AI内容安全赛道表现突出；保留清风卫AI安全。</t>
         </is>
       </c>
       <c r="E380" s="6" t="inlineStr">
@@ -11147,22 +11147,22 @@
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>PDF文档AI</t>
+          <t>AI办公Agent</t>
         </is>
       </c>
       <c r="B381" s="3" t="inlineStr">
         <is>
-          <t>688095</t>
+          <t>688111</t>
         </is>
       </c>
       <c r="C381" s="2" t="inlineStr">
         <is>
-          <t>福昕软件</t>
+          <t>金山办公</t>
         </is>
       </c>
       <c r="D381" s="2" t="inlineStr">
         <is>
-          <t>证据中强：公司核心仍是PDF/OFD版式文档软件，2025年营收高增并推进AI-Powered Research Agent、智能文档解析、结构化提取和私域知识库；主板块保留PDF文档AI。</t>
+          <t>证据强：2025年报披露WPS AI政务版、企业知识库、可信溯源和私有化部署等能力，WPS 365持续向企业级智能办公平台演进；企业知识库是AI办公Agent底座能力，合并到备注。</t>
         </is>
       </c>
       <c r="E381" s="6" t="inlineStr">
@@ -11174,22 +11174,22 @@
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>问财金融投研AI</t>
+          <t>PDF文档AI</t>
         </is>
       </c>
       <c r="B382" s="3" t="inlineStr">
         <is>
-          <t>300033</t>
+          <t>688095</t>
         </is>
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>同花顺</t>
+          <t>福昕软件</t>
         </is>
       </c>
       <c r="D382" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025财务决算披露公司持续加大AI研发、自研大模型并提升金融专业场景准确性，叠加营收和净利高增；AI变现依托问财/投研助手和金融信息服务，主线细化为问财金融投研AI。</t>
+          <t>证据中强：公司核心仍是PDF/OFD版式文档软件，2025年营收高增并推进AI-Powered Research Agent、智能文档解析、结构化提取和私域知识库；主板块保留PDF文档AI。</t>
         </is>
       </c>
       <c r="E382" s="6" t="inlineStr">
@@ -11201,22 +11201,22 @@
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>保险IT AI应用</t>
+          <t>问财金融投研AI</t>
         </is>
       </c>
       <c r="B383" s="3" t="inlineStr">
         <is>
-          <t>603927</t>
+          <t>300033</t>
         </is>
       </c>
       <c r="C383" s="2" t="inlineStr">
         <is>
-          <t>中科软</t>
+          <t>同花顺</t>
         </is>
       </c>
       <c r="D383" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司聚焦行业应用软件开发，保险IT解决方案市场占有率持续领先，并继续深耕保险、医疗卫生及政务等重点行业AI应用；主线保留保险IT AI应用，政务AI办公智能体并入备注不单列。</t>
+          <t>证据强：2025财务决算披露公司持续加大AI研发、自研大模型并提升金融专业场景准确性，叠加营收和净利高增；AI变现依托问财/投研助手和金融信息服务，主线细化为问财金融投研AI。</t>
         </is>
       </c>
       <c r="E383" s="6" t="inlineStr">
@@ -11228,22 +11228,22 @@
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>AI多媒体创作平台</t>
+          <t>保险IT AI应用</t>
         </is>
       </c>
       <c r="B384" s="3" t="inlineStr">
         <is>
-          <t>300624</t>
+          <t>603927</t>
         </is>
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>万兴科技</t>
+          <t>中科软</t>
         </is>
       </c>
       <c r="D384" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露万兴天幕2.0音视频多媒体大模型、AI漫剧/视频创作工作流，全年AI原生应用收入超1.3亿元、同比超90%；主板块由多媒体创作AI收敛为AI多媒体创作平台。</t>
+          <t>证据中强：2025年报披露公司聚焦行业应用软件开发，保险IT解决方案市场占有率持续领先，并继续深耕保险、医疗卫生及政务等重点行业AI应用；主线保留保险IT AI应用，政务AI办公智能体并入备注不单列。</t>
         </is>
       </c>
       <c r="E384" s="6" t="inlineStr">
@@ -11255,22 +11255,22 @@
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>AI+CAx工业设计软件</t>
+          <t>AI多媒体创作平台</t>
         </is>
       </c>
       <c r="B385" s="3" t="inlineStr">
         <is>
-          <t>688083</t>
+          <t>300624</t>
         </is>
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>中望软件</t>
+          <t>万兴科技</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司持续探索AI与CAx软件深度融合，ZWCAD 2026集成相似图形检索等AI功能并以API赋能生态；核心仍是研发设计类工业软件，主板块由工业设计AI细化为AI+CAx工业设计软件。</t>
+          <t>证据强：2025年报披露万兴天幕2.0音视频多媒体大模型、AI漫剧/视频创作工作流，全年AI原生应用收入超1.3亿元、同比超90%；主板块由多媒体创作AI收敛为AI多媒体创作平台。</t>
         </is>
       </c>
       <c r="E385" s="6" t="inlineStr">
@@ -11282,22 +11282,22 @@
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>物理AI工业仿真</t>
+          <t>AI+CAx工业设计软件</t>
         </is>
       </c>
       <c r="B386" s="3" t="inlineStr">
         <is>
-          <t>688507</t>
+          <t>688083</t>
         </is>
       </c>
       <c r="C386" s="2" t="inlineStr">
         <is>
-          <t>索辰科技</t>
+          <t>中望软件</t>
         </is>
       </c>
       <c r="D386" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司以CAE为核心并新增开物系列物理AI平台，物理AI聚焦工业场景机理建模与精准计算，产品矩阵从CAE延伸至工业软件全链条；主板块由工业仿真AI升级为物理AI工业仿真。</t>
+          <t>证据中强：2025年报披露公司持续探索AI与CAx软件深度融合，ZWCAD 2026集成相似图形检索等AI功能并以API赋能生态；核心仍是研发设计类工业软件，主板块由工业设计AI细化为AI+CAx工业设计软件。</t>
         </is>
       </c>
       <c r="E386" s="6" t="inlineStr">
@@ -11309,22 +11309,22 @@
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>流程工业AI</t>
+          <t>物理AI工业仿真</t>
         </is>
       </c>
       <c r="B387" s="3" t="inlineStr">
         <is>
-          <t>688777</t>
+          <t>688507</t>
         </is>
       </c>
       <c r="C387" s="2" t="inlineStr">
         <is>
-          <t>中控技术</t>
+          <t>索辰科技</t>
         </is>
       </c>
       <c r="D387" s="2" t="inlineStr">
         <is>
-          <t>证据强：公司持续深化All in AI战略，将AI能力融入流程工业控制、数据与场景体系；客户和控制系统部署基础集中在石化、化工、电力、冶金、制药等流程工业，主板块由工业AI收敛为流程工业AI。</t>
+          <t>证据强：2025年报披露公司以CAE为核心并新增开物系列物理AI平台，物理AI聚焦工业场景机理建模与精准计算，产品矩阵从CAE延伸至工业软件全链条；主板块由工业仿真AI升级为物理AI工业仿真。</t>
         </is>
       </c>
       <c r="E387" s="6" t="inlineStr">
@@ -11336,22 +11336,22 @@
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>激光加工AI工艺优化</t>
+          <t>流程工业AI</t>
         </is>
       </c>
       <c r="B388" s="3" t="inlineStr">
         <is>
-          <t>688188</t>
+          <t>688777</t>
         </is>
       </c>
       <c r="C388" s="2" t="inlineStr">
         <is>
-          <t>柏楚电子</t>
+          <t>中控技术</t>
         </is>
       </c>
       <c r="D388" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司在金属成型中基于自研AI模型实现切割断面自动采集与闭环工艺调试，并推进智能焊接、视觉识别和多机协同；主板块由工艺专家库细化为激光加工AI工艺优化。</t>
+          <t>证据强：公司持续深化All in AI战略，将AI能力融入流程工业控制、数据与场景体系；客户和控制系统部署基础集中在石化、化工、电力、冶金、制药等流程工业，主板块由工业AI收敛为流程工业AI。</t>
         </is>
       </c>
       <c r="E388" s="6" t="inlineStr">
@@ -11363,22 +11363,22 @@
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>AI分子砌块设计</t>
+          <t>激光加工AI工艺优化</t>
         </is>
       </c>
       <c r="B389" s="3" t="inlineStr">
         <is>
-          <t>300725</t>
+          <t>688188</t>
         </is>
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>药石科技</t>
+          <t>柏楚电子</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年投资者交流披露公司在前端分子砌块研发中应用AI生成8,000多万个新颖分子砌块，筛选后产品已陆续上线；核心仍是分子砌块+CDMO，主板块由AI分子砌块筛选细化为AI分子砌块设计。</t>
+          <t>证据强：2025年报披露公司在金属成型中基于自研AI模型实现切割断面自动采集与闭环工艺调试，并推进智能焊接、视觉识别和多机协同；主板块由工艺专家库细化为激光加工AI工艺优化。</t>
         </is>
       </c>
       <c r="E389" s="6" t="inlineStr">
@@ -11390,22 +11390,22 @@
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>AI片段分子库</t>
+          <t>AI分子砌块设计</t>
         </is>
       </c>
       <c r="B390" s="3" t="inlineStr">
         <is>
-          <t>688131</t>
+          <t>300725</t>
         </is>
       </c>
       <c r="C390" s="2" t="inlineStr">
         <is>
-          <t>皓元医药</t>
+          <t>药石科技</t>
         </is>
       </c>
       <c r="D390" s="2" t="inlineStr">
         <is>
-          <t>证据中：2025年报披露公司开发药物片段分子库，完成1万多种可用于药物筛选的小分子及类似物，并指出片段分子库结合人工智能大数据和实验筛选模型用于先导化合物发现；AI化合物库收敛为AI片段分子库。</t>
+          <t>证据中强：2025年投资者交流披露公司在前端分子砌块研发中应用AI生成8,000多万个新颖分子砌块，筛选后产品已陆续上线；核心仍是分子砌块+CDMO，主板块由AI分子砌块筛选细化为AI分子砌块设计。</t>
         </is>
       </c>
       <c r="E390" s="6" t="inlineStr">
@@ -11417,22 +11417,22 @@
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>AI药物发现</t>
+          <t>AI片段分子库</t>
         </is>
       </c>
       <c r="B391" s="3" t="inlineStr">
         <is>
-          <t>688222</t>
+          <t>688131</t>
         </is>
       </c>
       <c r="C391" s="2" t="inlineStr">
         <is>
-          <t>成都先导</t>
+          <t>皓元医药</t>
         </is>
       </c>
       <c r="D391" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以DEL技术为核心，并自主研发DEL+AI+自动化一体化分子优化平台HAILO，覆盖计算科学/AI数据分析与分子设计；主板块由AI制药收敛为AI药物发现。</t>
+          <t>证据中：2025年报披露公司开发药物片段分子库，完成1万多种可用于药物筛选的小分子及类似物，并指出片段分子库结合人工智能大数据和实验筛选模型用于先导化合物发现；AI化合物库收敛为AI片段分子库。</t>
         </is>
       </c>
       <c r="E391" s="6" t="inlineStr">
@@ -11444,22 +11444,22 @@
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>AI辅助药物设计</t>
+          <t>AI药物发现</t>
         </is>
       </c>
       <c r="B392" s="3" t="inlineStr">
         <is>
-          <t>301230</t>
+          <t>688222</t>
         </is>
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>泓博医药</t>
+          <t>成都先导</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
         <is>
-          <t>证据中强：2025年报披露公司以药物设计为核心驱动，在先导化合物发现阶段使用计算机/人工智能辅助药物设计，并覆盖靶点识别、虚拟筛选、结构预测、分子对接、分子动力学和ADME预测；AI是CRO/CDMO服务能力，不单列泛AI制药。</t>
+          <t>证据中强：2025年报披露公司以DEL技术为核心，并自主研发DEL+AI+自动化一体化分子优化平台HAILO，覆盖计算科学/AI数据分析与分子设计；主板块由AI制药收敛为AI药物发现。</t>
         </is>
       </c>
       <c r="E392" s="6" t="inlineStr">
@@ -11471,22 +11471,22 @@
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>AI患者追踪系统</t>
+          <t>AI辅助药物设计</t>
         </is>
       </c>
       <c r="B393" s="3" t="inlineStr">
         <is>
-          <t>300451</t>
+          <t>301230</t>
         </is>
       </c>
       <c r="C393" s="2" t="inlineStr">
         <is>
-          <t>创业慧康</t>
+          <t>泓博医药</t>
         </is>
       </c>
       <c r="D393" s="2" t="inlineStr">
         <is>
-          <t>证据中强但基本面承压：2025年报披露公司以AI技术创新驱动医疗场景落地，AI关键患者追踪系统APTS以医疗大模型为底座筛查高危患者并开展分级追踪；医疗大模型概念收敛为更具体的AI患者追踪系统。</t>
+          <t>证据中强：2025年报披露公司以药物设计为核心驱动，在先导化合物发现阶段使用计算机/人工智能辅助药物设计，并覆盖靶点识别、虚拟筛选、结构预测、分子对接、分子动力学和ADME预测；AI是CRO/CDMO服务能力，不单列泛AI制药。</t>
         </is>
       </c>
       <c r="E393" s="6" t="inlineStr">
@@ -11498,22 +11498,22 @@
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>AI医学影像设备</t>
+          <t>AI患者追踪系统</t>
         </is>
       </c>
       <c r="B394" s="3" t="inlineStr">
         <is>
-          <t>688271</t>
+          <t>300451</t>
         </is>
       </c>
       <c r="C394" s="2" t="inlineStr">
         <is>
-          <t>联影医疗</t>
+          <t>创业慧康</t>
         </is>
       </c>
       <c r="D394" s="2" t="inlineStr">
         <is>
-          <t>证据强：2025年报披露公司医学影像与放疗设备收入创新高，并推进设备+AI在医学影像诊疗和治疗场景落地，原生智能超声、光子计数CT、双宽体双源CT等高端产品放量；主板块保留医疗影像AI并细化为AI医学影像设备。</t>
+          <t>证据中强但基本面承压：2025年报披露公司以AI技术创新驱动医疗场景落地，AI关键患者追踪系统APTS以医疗大模型为底座筛查高危患者并开展分级追踪；医疗大模型概念收敛为更具体的AI患者追踪系统。</t>
         </is>
       </c>
       <c r="E394" s="6" t="inlineStr">
@@ -11525,22 +11525,22 @@
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
         <is>
-          <t>医疗信息化大模型</t>
+          <t>AI医学影像设备</t>
         </is>
       </c>
       <c r="B395" s="3" t="inlineStr">
         <is>
-          <t>300253</t>
+          <t>688271</t>
         </is>
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>卫宁健康</t>
+          <t>联影医疗</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
         <is>
-          <t>证据强但业绩承压：2025年报/半年报披露公司发布WiNGPT医疗大模型和WiNEX Copilot，覆盖文书生成、病历质控、诊中决策、报告解读、护理评估等场景，并在多家医疗机构部署；主线为医疗信息化大模型而非通用医疗AI。</t>
+          <t>证据强：2025年报披露公司医学影像与放疗设备收入创新高，并推进设备+AI在医学影像诊疗和治疗场景落地，原生智能超声、光子计数CT、双宽体双源CT等高端产品放量；主板块保留医疗影像AI并细化为AI医学影像设备。</t>
         </is>
       </c>
       <c r="E395" s="6" t="inlineStr">
@@ -11552,25 +11552,52 @@
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
+          <t>医疗信息化大模型</t>
+        </is>
+      </c>
+      <c r="B396" s="3" t="inlineStr">
+        <is>
+          <t>300253</t>
+        </is>
+      </c>
+      <c r="C396" s="2" t="inlineStr">
+        <is>
+          <t>卫宁健康</t>
+        </is>
+      </c>
+      <c r="D396" s="2" t="inlineStr">
+        <is>
+          <t>证据强但业绩承压：2025年报/半年报披露公司发布WiNGPT医疗大模型和WiNEX Copilot，覆盖文书生成、病历质控、诊中决策、报告解读、护理评估等场景，并在多家医疗机构部署；主线为医疗信息化大模型而非通用医疗AI。</t>
+        </is>
+      </c>
+      <c r="E396" s="6" t="inlineStr">
+        <is>
+          <t>已处理</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="2" t="inlineStr">
+        <is>
           <t>医学检验AI服务</t>
         </is>
       </c>
-      <c r="B396" s="3" t="inlineStr">
+      <c r="B397" s="3" t="inlineStr">
         <is>
           <t>603108</t>
         </is>
       </c>
-      <c r="C396" s="2" t="inlineStr">
+      <c r="C397" s="2" t="inlineStr">
         <is>
           <t>润达医疗</t>
         </is>
       </c>
-      <c r="D396" s="2" t="inlineStr">
+      <c r="D397" s="2" t="inlineStr">
         <is>
           <t>证据中强但业绩弱：2025年报披露公司推出大模型产品CDx良医晓慧，覆盖数据基座、医生助理和健康智能体，已在华西、南方、齐鲁等医院落地；核心仍是IVD流通/实验室服务，主板块由IVD检验AI细化为医学检验AI服务。</t>
         </is>
       </c>
-      <c r="E396" s="6" t="inlineStr">
+      <c r="E397" s="6" t="inlineStr">
         <is>
           <t>已处理</t>
         </is>

</xml_diff>